<commit_message>
Make direct NPD payment the baseline column and reference point
The direct-to-contractor block moves ahead of the 4dev platform block,
and all three delta columns now measure against it: platform, USN and
AUSN each show what they add over paying the contractor directly. The
planning block follows the same order.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019wo4Lmevz8VeqLa4QdqkBF
</commit_message>
<xml_diff>
--- a/СЗ_сравнение_схем_4dev_НПД_УСН_АУСН.xlsx
+++ b/СЗ_сравнение_схем_4dev_НПД_УСН_АУСН.xlsx
@@ -128,12 +128,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002E75B6"/>
+        <fgColor rgb="00548235"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00548235"/>
+        <fgColor rgb="002E75B6"/>
       </patternFill>
     </fill>
     <fill>
@@ -677,12 +677,12 @@
     <col width="12" customWidth="1" min="13" max="13"/>
     <col width="16" customWidth="1" min="14" max="14"/>
     <col width="18" customWidth="1" min="15" max="15"/>
-    <col width="15" customWidth="1" min="16" max="16"/>
-    <col width="17" customWidth="1" min="17" max="17"/>
-    <col width="13" customWidth="1" min="18" max="18"/>
-    <col width="18" customWidth="1" min="19" max="19"/>
+    <col width="13" customWidth="1" min="16" max="16"/>
+    <col width="16" customWidth="1" min="17" max="17"/>
+    <col width="15" customWidth="1" min="18" max="18"/>
+    <col width="17" customWidth="1" min="19" max="19"/>
     <col width="13" customWidth="1" min="20" max="20"/>
-    <col width="16" customWidth="1" min="21" max="21"/>
+    <col width="18" customWidth="1" min="21" max="21"/>
     <col width="14" customWidth="1" min="22" max="22"/>
     <col width="17" customWidth="1" min="23" max="23"/>
     <col width="14" customWidth="1" min="24" max="24"/>
@@ -874,17 +874,17 @@
       </c>
       <c r="P11" s="8" t="inlineStr">
         <is>
+          <t>Напрямую самозанятому (НПД)</t>
+        </is>
+      </c>
+      <c r="Q11" s="9" t="n"/>
+      <c r="R11" s="10" t="inlineStr">
+        <is>
           <t>Через площадку 4dev</t>
         </is>
       </c>
-      <c r="Q11" s="9" t="n"/>
-      <c r="R11" s="9" t="n"/>
-      <c r="S11" s="9" t="n"/>
-      <c r="T11" s="10" t="inlineStr">
-        <is>
-          <t>Напрямую самозанятому (НПД)</t>
-        </is>
-      </c>
+      <c r="S11" s="11" t="n"/>
+      <c r="T11" s="11" t="n"/>
       <c r="U11" s="11" t="n"/>
       <c r="V11" s="12" t="inlineStr">
         <is>
@@ -900,7 +900,7 @@
       <c r="Y11" s="15" t="n"/>
       <c r="Z11" s="16" t="inlineStr">
         <is>
-          <t>Разница, в месяц</t>
+          <t>Разница к НПД, в месяц</t>
         </is>
       </c>
       <c r="AA11" s="17" t="n"/>
@@ -924,34 +924,34 @@
       <c r="O12" s="18" t="n"/>
       <c r="P12" s="19" t="inlineStr">
         <is>
+          <t>НПД</t>
+        </is>
+      </c>
+      <c r="Q12" s="19" t="inlineStr">
+        <is>
+          <t>Выплата в месяц</t>
+        </is>
+      </c>
+      <c r="R12" s="20" t="inlineStr">
+        <is>
           <t>Комиссия 4dev 3%</t>
         </is>
       </c>
-      <c r="Q12" s="19" t="inlineStr">
+      <c r="S12" s="20" t="inlineStr">
         <is>
           <t>Сбор ЮЛ Сингапура 2,5%</t>
         </is>
       </c>
-      <c r="R12" s="19" t="inlineStr">
+      <c r="T12" s="20" t="inlineStr">
         <is>
           <t>НПД</t>
         </is>
       </c>
-      <c r="S12" s="19" t="inlineStr">
+      <c r="U12" s="20" t="inlineStr">
         <is>
           <t>ИТОГО к оплате в месяц</t>
         </is>
       </c>
-      <c r="T12" s="20" t="inlineStr">
-        <is>
-          <t>НПД</t>
-        </is>
-      </c>
-      <c r="U12" s="20" t="inlineStr">
-        <is>
-          <t>Выплата в месяц</t>
-        </is>
-      </c>
       <c r="V12" s="21" t="inlineStr">
         <is>
           <t>Налог в месяц</t>
@@ -974,17 +974,17 @@
       </c>
       <c r="Z12" s="23" t="inlineStr">
         <is>
-          <t>УСН − 4dev</t>
+          <t>4dev − НПД</t>
         </is>
       </c>
       <c r="AA12" s="23" t="inlineStr">
         <is>
-          <t>АУСН − 4dev</t>
+          <t>УСН − НПД</t>
         </is>
       </c>
       <c r="AB12" s="23" t="inlineStr">
         <is>
-          <t>АУСН − УСН</t>
+          <t>АУСН − НПД</t>
         </is>
       </c>
     </row>
@@ -1083,19 +1083,19 @@
         <v/>
       </c>
       <c r="P14" s="30">
+        <f>IF($AD14=0,0,O14/(1-$AD14)-O14)</f>
+        <v/>
+      </c>
+      <c r="Q14" s="31">
+        <f>O14+P14</f>
+        <v/>
+      </c>
+      <c r="R14" s="30">
         <f>O14*$C$6</f>
         <v/>
       </c>
-      <c r="Q14" s="30">
+      <c r="S14" s="30">
         <f>O14/(1-$C$7)-O14</f>
-        <v/>
-      </c>
-      <c r="R14" s="30">
-        <f>IF($AD14=0,0,O14/(1-$AD14)-O14)</f>
-        <v/>
-      </c>
-      <c r="S14" s="31">
-        <f>O14+P14+Q14+R14</f>
         <v/>
       </c>
       <c r="T14" s="30">
@@ -1103,7 +1103,7 @@
         <v/>
       </c>
       <c r="U14" s="31">
-        <f>O14+T14</f>
+        <f>O14+R14+S14+T14</f>
         <v/>
       </c>
       <c r="V14" s="30">
@@ -1123,15 +1123,15 @@
         <v/>
       </c>
       <c r="Z14" s="32">
-        <f>W14-S14</f>
+        <f>U14-Q14</f>
         <v/>
       </c>
       <c r="AA14" s="32">
-        <f>Y14-S14</f>
+        <f>W14-Q14</f>
         <v/>
       </c>
       <c r="AB14" s="32">
-        <f>Y14-W14</f>
+        <f>Y14-Q14</f>
         <v/>
       </c>
       <c r="AD14" s="33" t="n">
@@ -1199,19 +1199,19 @@
         <v/>
       </c>
       <c r="P15" s="38">
+        <f>IF($AD15=0,0,O15/(1-$AD15)-O15)</f>
+        <v/>
+      </c>
+      <c r="Q15" s="39">
+        <f>O15+P15</f>
+        <v/>
+      </c>
+      <c r="R15" s="38">
         <f>O15*$C$6</f>
         <v/>
       </c>
-      <c r="Q15" s="38">
+      <c r="S15" s="38">
         <f>O15/(1-$C$7)-O15</f>
-        <v/>
-      </c>
-      <c r="R15" s="38">
-        <f>IF($AD15=0,0,O15/(1-$AD15)-O15)</f>
-        <v/>
-      </c>
-      <c r="S15" s="39">
-        <f>O15+P15+Q15+R15</f>
         <v/>
       </c>
       <c r="T15" s="38">
@@ -1219,7 +1219,7 @@
         <v/>
       </c>
       <c r="U15" s="39">
-        <f>O15+T15</f>
+        <f>O15+R15+S15+T15</f>
         <v/>
       </c>
       <c r="V15" s="38">
@@ -1239,15 +1239,15 @@
         <v/>
       </c>
       <c r="Z15" s="40">
-        <f>W15-S15</f>
+        <f>U15-Q15</f>
         <v/>
       </c>
       <c r="AA15" s="40">
-        <f>Y15-S15</f>
+        <f>W15-Q15</f>
         <v/>
       </c>
       <c r="AB15" s="40">
-        <f>Y15-W15</f>
+        <f>Y15-Q15</f>
         <v/>
       </c>
       <c r="AD15" s="33" t="n">
@@ -1315,19 +1315,19 @@
         <v/>
       </c>
       <c r="P16" s="30">
+        <f>IF($AD16=0,0,O16/(1-$AD16)-O16)</f>
+        <v/>
+      </c>
+      <c r="Q16" s="31">
+        <f>O16+P16</f>
+        <v/>
+      </c>
+      <c r="R16" s="30">
         <f>O16*$C$6</f>
         <v/>
       </c>
-      <c r="Q16" s="30">
+      <c r="S16" s="30">
         <f>O16/(1-$C$7)-O16</f>
-        <v/>
-      </c>
-      <c r="R16" s="30">
-        <f>IF($AD16=0,0,O16/(1-$AD16)-O16)</f>
-        <v/>
-      </c>
-      <c r="S16" s="31">
-        <f>O16+P16+Q16+R16</f>
         <v/>
       </c>
       <c r="T16" s="30">
@@ -1335,7 +1335,7 @@
         <v/>
       </c>
       <c r="U16" s="31">
-        <f>O16+T16</f>
+        <f>O16+R16+S16+T16</f>
         <v/>
       </c>
       <c r="V16" s="30">
@@ -1355,15 +1355,15 @@
         <v/>
       </c>
       <c r="Z16" s="32">
-        <f>W16-S16</f>
+        <f>U16-Q16</f>
         <v/>
       </c>
       <c r="AA16" s="32">
-        <f>Y16-S16</f>
+        <f>W16-Q16</f>
         <v/>
       </c>
       <c r="AB16" s="32">
-        <f>Y16-W16</f>
+        <f>Y16-Q16</f>
         <v/>
       </c>
       <c r="AD16" s="33" t="n">
@@ -1431,19 +1431,19 @@
         <v/>
       </c>
       <c r="P17" s="38">
+        <f>IF($AD17=0,0,O17/(1-$AD17)-O17)</f>
+        <v/>
+      </c>
+      <c r="Q17" s="39">
+        <f>O17+P17</f>
+        <v/>
+      </c>
+      <c r="R17" s="38">
         <f>O17*$C$6</f>
         <v/>
       </c>
-      <c r="Q17" s="38">
+      <c r="S17" s="38">
         <f>O17/(1-$C$7)-O17</f>
-        <v/>
-      </c>
-      <c r="R17" s="38">
-        <f>IF($AD17=0,0,O17/(1-$AD17)-O17)</f>
-        <v/>
-      </c>
-      <c r="S17" s="39">
-        <f>O17+P17+Q17+R17</f>
         <v/>
       </c>
       <c r="T17" s="38">
@@ -1451,7 +1451,7 @@
         <v/>
       </c>
       <c r="U17" s="39">
-        <f>O17+T17</f>
+        <f>O17+R17+S17+T17</f>
         <v/>
       </c>
       <c r="V17" s="38">
@@ -1471,15 +1471,15 @@
         <v/>
       </c>
       <c r="Z17" s="40">
-        <f>W17-S17</f>
+        <f>U17-Q17</f>
         <v/>
       </c>
       <c r="AA17" s="40">
-        <f>Y17-S17</f>
+        <f>W17-Q17</f>
         <v/>
       </c>
       <c r="AB17" s="40">
-        <f>Y17-W17</f>
+        <f>Y17-Q17</f>
         <v/>
       </c>
       <c r="AD17" s="33" t="n">
@@ -1547,19 +1547,19 @@
         <v/>
       </c>
       <c r="P18" s="30">
+        <f>IF($AD18=0,0,O18/(1-$AD18)-O18)</f>
+        <v/>
+      </c>
+      <c r="Q18" s="31">
+        <f>O18+P18</f>
+        <v/>
+      </c>
+      <c r="R18" s="30">
         <f>O18*$C$6</f>
         <v/>
       </c>
-      <c r="Q18" s="30">
+      <c r="S18" s="30">
         <f>O18/(1-$C$7)-O18</f>
-        <v/>
-      </c>
-      <c r="R18" s="30">
-        <f>IF($AD18=0,0,O18/(1-$AD18)-O18)</f>
-        <v/>
-      </c>
-      <c r="S18" s="31">
-        <f>O18+P18+Q18+R18</f>
         <v/>
       </c>
       <c r="T18" s="30">
@@ -1567,7 +1567,7 @@
         <v/>
       </c>
       <c r="U18" s="31">
-        <f>O18+T18</f>
+        <f>O18+R18+S18+T18</f>
         <v/>
       </c>
       <c r="V18" s="30">
@@ -1587,15 +1587,15 @@
         <v/>
       </c>
       <c r="Z18" s="32">
-        <f>W18-S18</f>
+        <f>U18-Q18</f>
         <v/>
       </c>
       <c r="AA18" s="32">
-        <f>Y18-S18</f>
+        <f>W18-Q18</f>
         <v/>
       </c>
       <c r="AB18" s="32">
-        <f>Y18-W18</f>
+        <f>Y18-Q18</f>
         <v/>
       </c>
       <c r="AD18" s="33" t="n">
@@ -1663,19 +1663,19 @@
         <v/>
       </c>
       <c r="P19" s="38">
+        <f>IF($AD19=0,0,O19/(1-$AD19)-O19)</f>
+        <v/>
+      </c>
+      <c r="Q19" s="39">
+        <f>O19+P19</f>
+        <v/>
+      </c>
+      <c r="R19" s="38">
         <f>O19*$C$6</f>
         <v/>
       </c>
-      <c r="Q19" s="38">
+      <c r="S19" s="38">
         <f>O19/(1-$C$7)-O19</f>
-        <v/>
-      </c>
-      <c r="R19" s="38">
-        <f>IF($AD19=0,0,O19/(1-$AD19)-O19)</f>
-        <v/>
-      </c>
-      <c r="S19" s="39">
-        <f>O19+P19+Q19+R19</f>
         <v/>
       </c>
       <c r="T19" s="38">
@@ -1683,7 +1683,7 @@
         <v/>
       </c>
       <c r="U19" s="39">
-        <f>O19+T19</f>
+        <f>O19+R19+S19+T19</f>
         <v/>
       </c>
       <c r="V19" s="38">
@@ -1703,15 +1703,15 @@
         <v/>
       </c>
       <c r="Z19" s="40">
-        <f>W19-S19</f>
+        <f>U19-Q19</f>
         <v/>
       </c>
       <c r="AA19" s="40">
-        <f>Y19-S19</f>
+        <f>W19-Q19</f>
         <v/>
       </c>
       <c r="AB19" s="40">
-        <f>Y19-W19</f>
+        <f>Y19-Q19</f>
         <v/>
       </c>
       <c r="AD19" s="33" t="n">
@@ -1779,19 +1779,19 @@
         <v/>
       </c>
       <c r="P20" s="30">
+        <f>IF($AD20=0,0,O20/(1-$AD20)-O20)</f>
+        <v/>
+      </c>
+      <c r="Q20" s="31">
+        <f>O20+P20</f>
+        <v/>
+      </c>
+      <c r="R20" s="30">
         <f>O20*$C$6</f>
         <v/>
       </c>
-      <c r="Q20" s="30">
+      <c r="S20" s="30">
         <f>O20/(1-$C$7)-O20</f>
-        <v/>
-      </c>
-      <c r="R20" s="30">
-        <f>IF($AD20=0,0,O20/(1-$AD20)-O20)</f>
-        <v/>
-      </c>
-      <c r="S20" s="31">
-        <f>O20+P20+Q20+R20</f>
         <v/>
       </c>
       <c r="T20" s="30">
@@ -1799,7 +1799,7 @@
         <v/>
       </c>
       <c r="U20" s="31">
-        <f>O20+T20</f>
+        <f>O20+R20+S20+T20</f>
         <v/>
       </c>
       <c r="V20" s="30">
@@ -1819,15 +1819,15 @@
         <v/>
       </c>
       <c r="Z20" s="32">
-        <f>W20-S20</f>
+        <f>U20-Q20</f>
         <v/>
       </c>
       <c r="AA20" s="32">
-        <f>Y20-S20</f>
+        <f>W20-Q20</f>
         <v/>
       </c>
       <c r="AB20" s="32">
-        <f>Y20-W20</f>
+        <f>Y20-Q20</f>
         <v/>
       </c>
       <c r="AD20" s="33" t="n">
@@ -1895,19 +1895,19 @@
         <v/>
       </c>
       <c r="P21" s="38">
+        <f>IF($AD21=0,0,O21/(1-$AD21)-O21)</f>
+        <v/>
+      </c>
+      <c r="Q21" s="39">
+        <f>O21+P21</f>
+        <v/>
+      </c>
+      <c r="R21" s="38">
         <f>O21*$C$6</f>
         <v/>
       </c>
-      <c r="Q21" s="38">
+      <c r="S21" s="38">
         <f>O21/(1-$C$7)-O21</f>
-        <v/>
-      </c>
-      <c r="R21" s="38">
-        <f>IF($AD21=0,0,O21/(1-$AD21)-O21)</f>
-        <v/>
-      </c>
-      <c r="S21" s="39">
-        <f>O21+P21+Q21+R21</f>
         <v/>
       </c>
       <c r="T21" s="38">
@@ -1915,7 +1915,7 @@
         <v/>
       </c>
       <c r="U21" s="39">
-        <f>O21+T21</f>
+        <f>O21+R21+S21+T21</f>
         <v/>
       </c>
       <c r="V21" s="38">
@@ -1935,15 +1935,15 @@
         <v/>
       </c>
       <c r="Z21" s="40">
-        <f>W21-S21</f>
+        <f>U21-Q21</f>
         <v/>
       </c>
       <c r="AA21" s="40">
-        <f>Y21-S21</f>
+        <f>W21-Q21</f>
         <v/>
       </c>
       <c r="AB21" s="40">
-        <f>Y21-W21</f>
+        <f>Y21-Q21</f>
         <v/>
       </c>
       <c r="AD21" s="33" t="n">
@@ -2011,19 +2011,19 @@
         <v/>
       </c>
       <c r="P22" s="30">
+        <f>IF($AD22=0,0,O22/(1-$AD22)-O22)</f>
+        <v/>
+      </c>
+      <c r="Q22" s="31">
+        <f>O22+P22</f>
+        <v/>
+      </c>
+      <c r="R22" s="30">
         <f>O22*$C$6</f>
         <v/>
       </c>
-      <c r="Q22" s="30">
+      <c r="S22" s="30">
         <f>O22/(1-$C$7)-O22</f>
-        <v/>
-      </c>
-      <c r="R22" s="30">
-        <f>IF($AD22=0,0,O22/(1-$AD22)-O22)</f>
-        <v/>
-      </c>
-      <c r="S22" s="31">
-        <f>O22+P22+Q22+R22</f>
         <v/>
       </c>
       <c r="T22" s="30">
@@ -2031,7 +2031,7 @@
         <v/>
       </c>
       <c r="U22" s="31">
-        <f>O22+T22</f>
+        <f>O22+R22+S22+T22</f>
         <v/>
       </c>
       <c r="V22" s="30">
@@ -2051,15 +2051,15 @@
         <v/>
       </c>
       <c r="Z22" s="32">
-        <f>W22-S22</f>
+        <f>U22-Q22</f>
         <v/>
       </c>
       <c r="AA22" s="32">
-        <f>Y22-S22</f>
+        <f>W22-Q22</f>
         <v/>
       </c>
       <c r="AB22" s="32">
-        <f>Y22-W22</f>
+        <f>Y22-Q22</f>
         <v/>
       </c>
       <c r="AD22" s="33" t="n">
@@ -2127,19 +2127,19 @@
         <v/>
       </c>
       <c r="P23" s="38">
+        <f>IF($AD23=0,0,O23/(1-$AD23)-O23)</f>
+        <v/>
+      </c>
+      <c r="Q23" s="39">
+        <f>O23+P23</f>
+        <v/>
+      </c>
+      <c r="R23" s="38">
         <f>O23*$C$6</f>
         <v/>
       </c>
-      <c r="Q23" s="38">
+      <c r="S23" s="38">
         <f>O23/(1-$C$7)-O23</f>
-        <v/>
-      </c>
-      <c r="R23" s="38">
-        <f>IF($AD23=0,0,O23/(1-$AD23)-O23)</f>
-        <v/>
-      </c>
-      <c r="S23" s="39">
-        <f>O23+P23+Q23+R23</f>
         <v/>
       </c>
       <c r="T23" s="38">
@@ -2147,7 +2147,7 @@
         <v/>
       </c>
       <c r="U23" s="39">
-        <f>O23+T23</f>
+        <f>O23+R23+S23+T23</f>
         <v/>
       </c>
       <c r="V23" s="38">
@@ -2167,15 +2167,15 @@
         <v/>
       </c>
       <c r="Z23" s="40">
-        <f>W23-S23</f>
+        <f>U23-Q23</f>
         <v/>
       </c>
       <c r="AA23" s="40">
-        <f>Y23-S23</f>
+        <f>W23-Q23</f>
         <v/>
       </c>
       <c r="AB23" s="40">
-        <f>Y23-W23</f>
+        <f>Y23-Q23</f>
         <v/>
       </c>
       <c r="AD23" s="33" t="n">
@@ -2243,19 +2243,19 @@
         <v/>
       </c>
       <c r="P24" s="30">
+        <f>IF($AD24=0,0,O24/(1-$AD24)-O24)</f>
+        <v/>
+      </c>
+      <c r="Q24" s="31">
+        <f>O24+P24</f>
+        <v/>
+      </c>
+      <c r="R24" s="30">
         <f>O24*$C$6</f>
         <v/>
       </c>
-      <c r="Q24" s="30">
+      <c r="S24" s="30">
         <f>O24/(1-$C$7)-O24</f>
-        <v/>
-      </c>
-      <c r="R24" s="30">
-        <f>IF($AD24=0,0,O24/(1-$AD24)-O24)</f>
-        <v/>
-      </c>
-      <c r="S24" s="31">
-        <f>O24+P24+Q24+R24</f>
         <v/>
       </c>
       <c r="T24" s="30">
@@ -2263,7 +2263,7 @@
         <v/>
       </c>
       <c r="U24" s="31">
-        <f>O24+T24</f>
+        <f>O24+R24+S24+T24</f>
         <v/>
       </c>
       <c r="V24" s="30">
@@ -2283,15 +2283,15 @@
         <v/>
       </c>
       <c r="Z24" s="32">
-        <f>W24-S24</f>
+        <f>U24-Q24</f>
         <v/>
       </c>
       <c r="AA24" s="32">
-        <f>Y24-S24</f>
+        <f>W24-Q24</f>
         <v/>
       </c>
       <c r="AB24" s="32">
-        <f>Y24-W24</f>
+        <f>Y24-Q24</f>
         <v/>
       </c>
       <c r="AD24" s="33" t="n">
@@ -2359,19 +2359,19 @@
         <v/>
       </c>
       <c r="P25" s="38">
+        <f>IF($AD25=0,0,O25/(1-$AD25)-O25)</f>
+        <v/>
+      </c>
+      <c r="Q25" s="39">
+        <f>O25+P25</f>
+        <v/>
+      </c>
+      <c r="R25" s="38">
         <f>O25*$C$6</f>
         <v/>
       </c>
-      <c r="Q25" s="38">
+      <c r="S25" s="38">
         <f>O25/(1-$C$7)-O25</f>
-        <v/>
-      </c>
-      <c r="R25" s="38">
-        <f>IF($AD25=0,0,O25/(1-$AD25)-O25)</f>
-        <v/>
-      </c>
-      <c r="S25" s="39">
-        <f>O25+P25+Q25+R25</f>
         <v/>
       </c>
       <c r="T25" s="38">
@@ -2379,7 +2379,7 @@
         <v/>
       </c>
       <c r="U25" s="39">
-        <f>O25+T25</f>
+        <f>O25+R25+S25+T25</f>
         <v/>
       </c>
       <c r="V25" s="38">
@@ -2399,15 +2399,15 @@
         <v/>
       </c>
       <c r="Z25" s="40">
-        <f>W25-S25</f>
+        <f>U25-Q25</f>
         <v/>
       </c>
       <c r="AA25" s="40">
-        <f>Y25-S25</f>
+        <f>W25-Q25</f>
         <v/>
       </c>
       <c r="AB25" s="40">
-        <f>Y25-W25</f>
+        <f>Y25-Q25</f>
         <v/>
       </c>
       <c r="AD25" s="33" t="n">
@@ -2475,19 +2475,19 @@
         <v/>
       </c>
       <c r="P26" s="30">
+        <f>IF($AD26=0,0,O26/(1-$AD26)-O26)</f>
+        <v/>
+      </c>
+      <c r="Q26" s="31">
+        <f>O26+P26</f>
+        <v/>
+      </c>
+      <c r="R26" s="30">
         <f>O26*$C$6</f>
         <v/>
       </c>
-      <c r="Q26" s="30">
+      <c r="S26" s="30">
         <f>O26/(1-$C$7)-O26</f>
-        <v/>
-      </c>
-      <c r="R26" s="30">
-        <f>IF($AD26=0,0,O26/(1-$AD26)-O26)</f>
-        <v/>
-      </c>
-      <c r="S26" s="31">
-        <f>O26+P26+Q26+R26</f>
         <v/>
       </c>
       <c r="T26" s="30">
@@ -2495,7 +2495,7 @@
         <v/>
       </c>
       <c r="U26" s="31">
-        <f>O26+T26</f>
+        <f>O26+R26+S26+T26</f>
         <v/>
       </c>
       <c r="V26" s="30">
@@ -2515,15 +2515,15 @@
         <v/>
       </c>
       <c r="Z26" s="32">
-        <f>W26-S26</f>
+        <f>U26-Q26</f>
         <v/>
       </c>
       <c r="AA26" s="32">
-        <f>Y26-S26</f>
+        <f>W26-Q26</f>
         <v/>
       </c>
       <c r="AB26" s="32">
-        <f>Y26-W26</f>
+        <f>Y26-Q26</f>
         <v/>
       </c>
       <c r="AD26" s="33" t="n">
@@ -2591,19 +2591,19 @@
         <v/>
       </c>
       <c r="P27" s="38">
+        <f>IF($AD27=0,0,O27/(1-$AD27)-O27)</f>
+        <v/>
+      </c>
+      <c r="Q27" s="39">
+        <f>O27+P27</f>
+        <v/>
+      </c>
+      <c r="R27" s="38">
         <f>O27*$C$6</f>
         <v/>
       </c>
-      <c r="Q27" s="38">
+      <c r="S27" s="38">
         <f>O27/(1-$C$7)-O27</f>
-        <v/>
-      </c>
-      <c r="R27" s="38">
-        <f>IF($AD27=0,0,O27/(1-$AD27)-O27)</f>
-        <v/>
-      </c>
-      <c r="S27" s="39">
-        <f>O27+P27+Q27+R27</f>
         <v/>
       </c>
       <c r="T27" s="38">
@@ -2611,7 +2611,7 @@
         <v/>
       </c>
       <c r="U27" s="39">
-        <f>O27+T27</f>
+        <f>O27+R27+S27+T27</f>
         <v/>
       </c>
       <c r="V27" s="38">
@@ -2631,15 +2631,15 @@
         <v/>
       </c>
       <c r="Z27" s="40">
-        <f>W27-S27</f>
+        <f>U27-Q27</f>
         <v/>
       </c>
       <c r="AA27" s="40">
-        <f>Y27-S27</f>
+        <f>W27-Q27</f>
         <v/>
       </c>
       <c r="AB27" s="40">
-        <f>Y27-W27</f>
+        <f>Y27-Q27</f>
         <v/>
       </c>
       <c r="AD27" s="33" t="n">
@@ -2707,19 +2707,19 @@
         <v/>
       </c>
       <c r="P28" s="30">
+        <f>IF($AD28=0,0,O28/(1-$AD28)-O28)</f>
+        <v/>
+      </c>
+      <c r="Q28" s="31">
+        <f>O28+P28</f>
+        <v/>
+      </c>
+      <c r="R28" s="30">
         <f>O28*$C$6</f>
         <v/>
       </c>
-      <c r="Q28" s="30">
+      <c r="S28" s="30">
         <f>O28/(1-$C$7)-O28</f>
-        <v/>
-      </c>
-      <c r="R28" s="30">
-        <f>IF($AD28=0,0,O28/(1-$AD28)-O28)</f>
-        <v/>
-      </c>
-      <c r="S28" s="31">
-        <f>O28+P28+Q28+R28</f>
         <v/>
       </c>
       <c r="T28" s="30">
@@ -2727,7 +2727,7 @@
         <v/>
       </c>
       <c r="U28" s="31">
-        <f>O28+T28</f>
+        <f>O28+R28+S28+T28</f>
         <v/>
       </c>
       <c r="V28" s="30">
@@ -2747,15 +2747,15 @@
         <v/>
       </c>
       <c r="Z28" s="32">
-        <f>W28-S28</f>
+        <f>U28-Q28</f>
         <v/>
       </c>
       <c r="AA28" s="32">
-        <f>Y28-S28</f>
+        <f>W28-Q28</f>
         <v/>
       </c>
       <c r="AB28" s="32">
-        <f>Y28-W28</f>
+        <f>Y28-Q28</f>
         <v/>
       </c>
       <c r="AD28" s="33" t="n">
@@ -2951,19 +2951,19 @@
         <v/>
       </c>
       <c r="P32" s="30">
+        <f>IF($AD32=0,0,O32/(1-$AD32)-O32)</f>
+        <v/>
+      </c>
+      <c r="Q32" s="31">
+        <f>O32+P32</f>
+        <v/>
+      </c>
+      <c r="R32" s="30">
         <f>O32*$C$6</f>
         <v/>
       </c>
-      <c r="Q32" s="30">
+      <c r="S32" s="30">
         <f>O32/(1-$C$7)-O32</f>
-        <v/>
-      </c>
-      <c r="R32" s="30">
-        <f>IF($AD32=0,0,O32/(1-$AD32)-O32)</f>
-        <v/>
-      </c>
-      <c r="S32" s="31">
-        <f>O32+P32+Q32+R32</f>
         <v/>
       </c>
       <c r="T32" s="30">
@@ -2971,7 +2971,7 @@
         <v/>
       </c>
       <c r="U32" s="31">
-        <f>O32+T32</f>
+        <f>O32+R32+S32+T32</f>
         <v/>
       </c>
       <c r="V32" s="30">
@@ -2991,15 +2991,15 @@
         <v/>
       </c>
       <c r="Z32" s="32">
-        <f>W32-S32</f>
+        <f>U32-Q32</f>
         <v/>
       </c>
       <c r="AA32" s="32">
-        <f>Y32-S32</f>
+        <f>W32-Q32</f>
         <v/>
       </c>
       <c r="AB32" s="32">
-        <f>Y32-W32</f>
+        <f>Y32-Q32</f>
         <v/>
       </c>
       <c r="AD32" s="33" t="n">
@@ -3067,19 +3067,19 @@
         <v/>
       </c>
       <c r="P33" s="38">
+        <f>IF($AD33=0,0,O33/(1-$AD33)-O33)</f>
+        <v/>
+      </c>
+      <c r="Q33" s="39">
+        <f>O33+P33</f>
+        <v/>
+      </c>
+      <c r="R33" s="38">
         <f>O33*$C$6</f>
         <v/>
       </c>
-      <c r="Q33" s="38">
+      <c r="S33" s="38">
         <f>O33/(1-$C$7)-O33</f>
-        <v/>
-      </c>
-      <c r="R33" s="38">
-        <f>IF($AD33=0,0,O33/(1-$AD33)-O33)</f>
-        <v/>
-      </c>
-      <c r="S33" s="39">
-        <f>O33+P33+Q33+R33</f>
         <v/>
       </c>
       <c r="T33" s="38">
@@ -3087,7 +3087,7 @@
         <v/>
       </c>
       <c r="U33" s="39">
-        <f>O33+T33</f>
+        <f>O33+R33+S33+T33</f>
         <v/>
       </c>
       <c r="V33" s="38">
@@ -3107,15 +3107,15 @@
         <v/>
       </c>
       <c r="Z33" s="40">
-        <f>W33-S33</f>
+        <f>U33-Q33</f>
         <v/>
       </c>
       <c r="AA33" s="40">
-        <f>Y33-S33</f>
+        <f>W33-Q33</f>
         <v/>
       </c>
       <c r="AB33" s="40">
-        <f>Y33-W33</f>
+        <f>Y33-Q33</f>
         <v/>
       </c>
       <c r="AD33" s="33" t="n">
@@ -3183,19 +3183,19 @@
         <v/>
       </c>
       <c r="P34" s="30">
+        <f>IF($AD34=0,0,O34/(1-$AD34)-O34)</f>
+        <v/>
+      </c>
+      <c r="Q34" s="31">
+        <f>O34+P34</f>
+        <v/>
+      </c>
+      <c r="R34" s="30">
         <f>O34*$C$6</f>
         <v/>
       </c>
-      <c r="Q34" s="30">
+      <c r="S34" s="30">
         <f>O34/(1-$C$7)-O34</f>
-        <v/>
-      </c>
-      <c r="R34" s="30">
-        <f>IF($AD34=0,0,O34/(1-$AD34)-O34)</f>
-        <v/>
-      </c>
-      <c r="S34" s="31">
-        <f>O34+P34+Q34+R34</f>
         <v/>
       </c>
       <c r="T34" s="30">
@@ -3203,7 +3203,7 @@
         <v/>
       </c>
       <c r="U34" s="31">
-        <f>O34+T34</f>
+        <f>O34+R34+S34+T34</f>
         <v/>
       </c>
       <c r="V34" s="30">
@@ -3223,15 +3223,15 @@
         <v/>
       </c>
       <c r="Z34" s="32">
-        <f>W34-S34</f>
+        <f>U34-Q34</f>
         <v/>
       </c>
       <c r="AA34" s="32">
-        <f>Y34-S34</f>
+        <f>W34-Q34</f>
         <v/>
       </c>
       <c r="AB34" s="32">
-        <f>Y34-W34</f>
+        <f>Y34-Q34</f>
         <v/>
       </c>
       <c r="AD34" s="33" t="n">
@@ -3299,19 +3299,19 @@
         <v/>
       </c>
       <c r="P35" s="38">
+        <f>IF($AD35=0,0,O35/(1-$AD35)-O35)</f>
+        <v/>
+      </c>
+      <c r="Q35" s="39">
+        <f>O35+P35</f>
+        <v/>
+      </c>
+      <c r="R35" s="38">
         <f>O35*$C$6</f>
         <v/>
       </c>
-      <c r="Q35" s="38">
+      <c r="S35" s="38">
         <f>O35/(1-$C$7)-O35</f>
-        <v/>
-      </c>
-      <c r="R35" s="38">
-        <f>IF($AD35=0,0,O35/(1-$AD35)-O35)</f>
-        <v/>
-      </c>
-      <c r="S35" s="39">
-        <f>O35+P35+Q35+R35</f>
         <v/>
       </c>
       <c r="T35" s="38">
@@ -3319,7 +3319,7 @@
         <v/>
       </c>
       <c r="U35" s="39">
-        <f>O35+T35</f>
+        <f>O35+R35+S35+T35</f>
         <v/>
       </c>
       <c r="V35" s="38">
@@ -3339,15 +3339,15 @@
         <v/>
       </c>
       <c r="Z35" s="40">
-        <f>W35-S35</f>
+        <f>U35-Q35</f>
         <v/>
       </c>
       <c r="AA35" s="40">
-        <f>Y35-S35</f>
+        <f>W35-Q35</f>
         <v/>
       </c>
       <c r="AB35" s="40">
-        <f>Y35-W35</f>
+        <f>Y35-Q35</f>
         <v/>
       </c>
       <c r="AD35" s="33" t="n">
@@ -3543,19 +3543,19 @@
         <v/>
       </c>
       <c r="P39" s="30">
+        <f>IF($AD39=0,0,O39/(1-$AD39)-O39)</f>
+        <v/>
+      </c>
+      <c r="Q39" s="31">
+        <f>O39+P39</f>
+        <v/>
+      </c>
+      <c r="R39" s="30">
         <f>O39*$C$6</f>
         <v/>
       </c>
-      <c r="Q39" s="30">
+      <c r="S39" s="30">
         <f>O39/(1-$C$7)-O39</f>
-        <v/>
-      </c>
-      <c r="R39" s="30">
-        <f>IF($AD39=0,0,O39/(1-$AD39)-O39)</f>
-        <v/>
-      </c>
-      <c r="S39" s="31">
-        <f>O39+P39+Q39+R39</f>
         <v/>
       </c>
       <c r="T39" s="30">
@@ -3563,7 +3563,7 @@
         <v/>
       </c>
       <c r="U39" s="31">
-        <f>O39+T39</f>
+        <f>O39+R39+S39+T39</f>
         <v/>
       </c>
       <c r="V39" s="30">
@@ -3583,15 +3583,15 @@
         <v/>
       </c>
       <c r="Z39" s="32">
-        <f>W39-S39</f>
+        <f>U39-Q39</f>
         <v/>
       </c>
       <c r="AA39" s="32">
-        <f>Y39-S39</f>
+        <f>W39-Q39</f>
         <v/>
       </c>
       <c r="AB39" s="32">
-        <f>Y39-W39</f>
+        <f>Y39-Q39</f>
         <v/>
       </c>
       <c r="AD39" s="33" t="n">
@@ -3806,24 +3806,24 @@
       </c>
       <c r="C45" s="7" t="inlineStr">
         <is>
+          <t>Напрямую: месяц</t>
+        </is>
+      </c>
+      <c r="D45" s="7" t="inlineStr">
+        <is>
+          <t>Напрямую: год</t>
+        </is>
+      </c>
+      <c r="E45" s="7" t="inlineStr">
+        <is>
           <t>4dev: месяц</t>
         </is>
       </c>
-      <c r="D45" s="7" t="inlineStr">
+      <c r="F45" s="7" t="inlineStr">
         <is>
           <t>4dev: год</t>
         </is>
       </c>
-      <c r="E45" s="7" t="inlineStr">
-        <is>
-          <t>Напрямую: месяц</t>
-        </is>
-      </c>
-      <c r="F45" s="7" t="inlineStr">
-        <is>
-          <t>Напрямую: год</t>
-        </is>
-      </c>
       <c r="G45" s="7" t="inlineStr">
         <is>
           <t>УСН 7%: месяц</t>
@@ -3846,12 +3846,17 @@
       </c>
       <c r="K45" s="7" t="inlineStr">
         <is>
-          <t>УСН − 4dev за год</t>
+          <t>4dev − НПД за год</t>
         </is>
       </c>
       <c r="L45" s="7" t="inlineStr">
         <is>
-          <t>АУСН − 4dev за год</t>
+          <t>УСН − НПД за год</t>
+        </is>
+      </c>
+      <c r="M45" s="7" t="inlineStr">
+        <is>
+          <t>АУСН − НПД за год</t>
         </is>
       </c>
     </row>
@@ -3865,11 +3870,11 @@
         <v>15</v>
       </c>
       <c r="C46" s="50">
-        <f>S29</f>
+        <f>Q29</f>
         <v/>
       </c>
       <c r="D46" s="51">
-        <f>S29*12</f>
+        <f>Q29*12</f>
         <v/>
       </c>
       <c r="E46" s="50">
@@ -3904,6 +3909,10 @@
         <f>AA29*12</f>
         <v/>
       </c>
+      <c r="M46" s="51">
+        <f>AB29*12</f>
+        <v/>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="48" t="inlineStr">
@@ -3915,11 +3924,11 @@
         <v>4</v>
       </c>
       <c r="C47" s="50">
-        <f>S36</f>
+        <f>Q36</f>
         <v/>
       </c>
       <c r="D47" s="51">
-        <f>S36*12</f>
+        <f>Q36*12</f>
         <v/>
       </c>
       <c r="E47" s="50">
@@ -3954,6 +3963,10 @@
         <f>AA36*12</f>
         <v/>
       </c>
+      <c r="M47" s="51">
+        <f>AB36*12</f>
+        <v/>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="48" t="inlineStr">
@@ -3965,11 +3978,11 @@
         <v>1</v>
       </c>
       <c r="C48" s="50">
-        <f>S40</f>
+        <f>Q40</f>
         <v/>
       </c>
       <c r="D48" s="51">
-        <f>S40*12</f>
+        <f>Q40*12</f>
         <v/>
       </c>
       <c r="E48" s="50">
@@ -4004,6 +4017,10 @@
         <f>AA40*12</f>
         <v/>
       </c>
+      <c r="M48" s="51">
+        <f>AB40*12</f>
+        <v/>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="52" t="inlineStr">
@@ -4015,11 +4032,11 @@
         <v>20</v>
       </c>
       <c r="C49" s="54">
-        <f>S42</f>
+        <f>Q42</f>
         <v/>
       </c>
       <c r="D49" s="54">
-        <f>S42*12</f>
+        <f>Q42*12</f>
         <v/>
       </c>
       <c r="E49" s="54">
@@ -4054,6 +4071,10 @@
         <f>AA42*12</f>
         <v/>
       </c>
+      <c r="M49" s="54">
+        <f>AB42*12</f>
+        <v/>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="55" t="inlineStr">
@@ -4079,7 +4100,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>3. «Напрямую самозанятому» — та же работа без площадки: на руки + НПД, без комиссии и сбора. Разница с блоком 4dev = стоимость площадки.</t>
+          <t>3. «Напрямую самозанятому» — базовый вариант: на руки + НПД, без комиссии и сбора. Все разницы в таблице считаются именно от него.</t>
         </is>
       </c>
     </row>
@@ -4134,14 +4155,14 @@
     <mergeCell ref="H11:H12"/>
     <mergeCell ref="J11:J12"/>
     <mergeCell ref="K11:K12"/>
+    <mergeCell ref="P11:Q11"/>
     <mergeCell ref="C11:C12"/>
+    <mergeCell ref="R11:U11"/>
     <mergeCell ref="E11:E12"/>
-    <mergeCell ref="T11:U11"/>
     <mergeCell ref="V11:W11"/>
     <mergeCell ref="O11:O12"/>
     <mergeCell ref="F11:F12"/>
     <mergeCell ref="L11:L12"/>
-    <mergeCell ref="P11:S11"/>
     <mergeCell ref="N11:N12"/>
     <mergeCell ref="Z11:AB11"/>
     <mergeCell ref="G11:G12"/>

</xml_diff>

<commit_message>
Apply client-confirmed 2025 totals and add Shultyaeva to the roster
Fourteen 2025 figures supplied by the client replace the partial sums
assembled from payment rows, correcting Kuzmina, Lukyanova, Tupiko,
Repetenko and Nurullina by a wide margin. Confirmed cells are shaded
green, leaving the shrinking set of still-uncertain ones in amber.
Shultyaeva joins the list as the twenty-first person.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019wo4Lmevz8VeqLa4QdqkBF
</commit_message>
<xml_diff>
--- a/СЗ_сравнение_схем_4dev_НПД_УСН_АУСН.xlsx
+++ b/СЗ_сравнение_схем_4dev_НПД_УСН_АУСН.xlsx
@@ -40,12 +40,6 @@
     </font>
     <font>
       <name val="Arial"/>
-      <i val="1"/>
-      <color rgb="00C55A11"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Arial"/>
       <b val="1"/>
       <sz val="10"/>
     </font>
@@ -76,6 +70,12 @@
       <b val="1"/>
       <color rgb="001F4E78"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00375623"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -121,7 +121,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="15">
+  <fills count="16">
     <fill>
       <patternFill/>
     </fill>
@@ -166,6 +166,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D9E1F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
     <fill>
@@ -226,92 +231,92 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="10" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="9" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="10" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="12" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="13" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="14" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="15" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="5" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="12" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="13" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="14" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="15" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="4" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="12" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="13" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="14" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="15" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="16" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="16" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="3" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="14" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="16" fillId="14" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="14" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="15" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="14" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="4" fillId="14" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="4" fillId="15" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="3" fillId="15" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="14" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="3" fillId="14" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -678,7 +683,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD63"/>
+  <dimension ref="A1:AD66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -727,26 +732,26 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Ячейки с оранжевой заливкой в столбцах 2022–2026 собраны по отдельным строкам выплат: годовая сводная по этим людям в выгрузку не попала, суммы могут быть занижены.</t>
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Зелёные ячейки — суммы за 2025 подтверждены заказчиком. Оранжевые — собраны по отдельным строкам выплат (годовая сводная по этим людям в выгрузку не попала), могут быть занижены.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>ДОПУЩЕНИЯ (синие ячейки — можно менять, всё пересчитается). Ставка НПД берётся по каждому человеку из столбца E.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>Выплат в 2026 (мес.)</t>
         </is>
       </c>
-      <c r="C5" s="6" t="n">
+      <c r="C5" s="5" t="n">
         <v>7</v>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -756,12 +761,12 @@
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>Комиссия платформы 4dev</t>
         </is>
       </c>
-      <c r="C6" s="7" t="n">
+      <c r="C6" s="6" t="n">
         <v>0.03</v>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -771,12 +776,12 @@
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>Сбор ЮЛ Сингапура</t>
         </is>
       </c>
-      <c r="C7" s="7" t="n">
+      <c r="C7" s="6" t="n">
         <v>0.025</v>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -786,12 +791,12 @@
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>Ставка УСН «доходы»</t>
         </is>
       </c>
-      <c r="C8" s="7" t="n">
+      <c r="C8" s="6" t="n">
         <v>0.07000000000000001</v>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -801,12 +806,12 @@
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>Ставка АУСН «доходы»</t>
         </is>
       </c>
-      <c r="C9" s="7" t="n">
+      <c r="C9" s="6" t="n">
         <v>0.08</v>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -816,275 +821,275 @@
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="A11" s="7" t="inlineStr">
         <is>
           <t>№</t>
         </is>
       </c>
-      <c r="B11" s="8" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>ФИО</t>
         </is>
       </c>
-      <c r="C11" s="8" t="inlineStr">
+      <c r="C11" s="7" t="inlineStr">
         <is>
           <t>Проект</t>
         </is>
       </c>
-      <c r="D11" s="8" t="inlineStr">
+      <c r="D11" s="7" t="inlineStr">
         <is>
           <t>ЮЛ</t>
         </is>
       </c>
-      <c r="E11" s="8" t="inlineStr">
+      <c r="E11" s="7" t="inlineStr">
         <is>
           <t>Ставка НПД</t>
         </is>
       </c>
-      <c r="F11" s="8" t="inlineStr">
+      <c r="F11" s="7" t="inlineStr">
         <is>
           <t>Статус</t>
         </is>
       </c>
-      <c r="G11" s="8" t="inlineStr">
+      <c r="G11" s="7" t="inlineStr">
         <is>
           <t>Период выплат</t>
         </is>
       </c>
-      <c r="H11" s="8" t="inlineStr">
+      <c r="H11" s="7" t="inlineStr">
         <is>
           <t>Лет</t>
         </is>
       </c>
-      <c r="I11" s="8" t="inlineStr">
+      <c r="I11" s="7" t="inlineStr">
         <is>
           <t>2022</t>
         </is>
       </c>
-      <c r="J11" s="8" t="inlineStr">
+      <c r="J11" s="7" t="inlineStr">
         <is>
           <t>2023</t>
         </is>
       </c>
-      <c r="K11" s="8" t="inlineStr">
+      <c r="K11" s="7" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="L11" s="8" t="inlineStr">
+      <c r="L11" s="7" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="M11" s="8" t="inlineStr">
+      <c r="M11" s="7" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="N11" s="8" t="inlineStr">
+      <c r="N11" s="7" t="inlineStr">
         <is>
           <t>Итого 2022–2026</t>
         </is>
       </c>
-      <c r="O11" s="8" t="inlineStr">
+      <c r="O11" s="7" t="inlineStr">
         <is>
           <t>Среднемес. на руки 2026</t>
         </is>
       </c>
-      <c r="P11" s="9" t="inlineStr">
+      <c r="P11" s="8" t="inlineStr">
         <is>
           <t>Напрямую самозанятому (НПД)</t>
         </is>
       </c>
-      <c r="Q11" s="10" t="n"/>
-      <c r="R11" s="11" t="inlineStr">
+      <c r="Q11" s="9" t="n"/>
+      <c r="R11" s="10" t="inlineStr">
         <is>
           <t>Через площадку 4dev</t>
         </is>
       </c>
-      <c r="S11" s="12" t="n"/>
-      <c r="T11" s="12" t="n"/>
-      <c r="U11" s="12" t="n"/>
-      <c r="V11" s="13" t="inlineStr">
+      <c r="S11" s="11" t="n"/>
+      <c r="T11" s="11" t="n"/>
+      <c r="U11" s="11" t="n"/>
+      <c r="V11" s="12" t="inlineStr">
         <is>
           <t>ИП на УСН 7%</t>
         </is>
       </c>
-      <c r="W11" s="14" t="n"/>
-      <c r="X11" s="15" t="inlineStr">
+      <c r="W11" s="13" t="n"/>
+      <c r="X11" s="14" t="inlineStr">
         <is>
           <t>ИП на АУСН 8%</t>
         </is>
       </c>
-      <c r="Y11" s="16" t="n"/>
-      <c r="Z11" s="17" t="inlineStr">
+      <c r="Y11" s="15" t="n"/>
+      <c r="Z11" s="16" t="inlineStr">
         <is>
           <t>Разница к НПД, в месяц</t>
         </is>
       </c>
-      <c r="AA11" s="18" t="n"/>
-      <c r="AB11" s="18" t="n"/>
+      <c r="AA11" s="17" t="n"/>
+      <c r="AB11" s="17" t="n"/>
     </row>
     <row r="12" ht="40" customHeight="1">
-      <c r="A12" s="19" t="n"/>
-      <c r="B12" s="19" t="n"/>
-      <c r="C12" s="19" t="n"/>
-      <c r="D12" s="19" t="n"/>
-      <c r="E12" s="19" t="n"/>
-      <c r="F12" s="19" t="n"/>
-      <c r="G12" s="19" t="n"/>
-      <c r="H12" s="19" t="n"/>
-      <c r="I12" s="19" t="n"/>
-      <c r="J12" s="19" t="n"/>
-      <c r="K12" s="19" t="n"/>
-      <c r="L12" s="19" t="n"/>
-      <c r="M12" s="19" t="n"/>
-      <c r="N12" s="19" t="n"/>
-      <c r="O12" s="19" t="n"/>
-      <c r="P12" s="20" t="inlineStr">
+      <c r="A12" s="18" t="n"/>
+      <c r="B12" s="18" t="n"/>
+      <c r="C12" s="18" t="n"/>
+      <c r="D12" s="18" t="n"/>
+      <c r="E12" s="18" t="n"/>
+      <c r="F12" s="18" t="n"/>
+      <c r="G12" s="18" t="n"/>
+      <c r="H12" s="18" t="n"/>
+      <c r="I12" s="18" t="n"/>
+      <c r="J12" s="18" t="n"/>
+      <c r="K12" s="18" t="n"/>
+      <c r="L12" s="18" t="n"/>
+      <c r="M12" s="18" t="n"/>
+      <c r="N12" s="18" t="n"/>
+      <c r="O12" s="18" t="n"/>
+      <c r="P12" s="19" t="inlineStr">
         <is>
           <t>НПД</t>
         </is>
       </c>
-      <c r="Q12" s="20" t="inlineStr">
+      <c r="Q12" s="19" t="inlineStr">
         <is>
           <t>Выплата в месяц</t>
         </is>
       </c>
-      <c r="R12" s="21" t="inlineStr">
+      <c r="R12" s="20" t="inlineStr">
         <is>
           <t>Комиссия 4dev 3%</t>
         </is>
       </c>
-      <c r="S12" s="21" t="inlineStr">
+      <c r="S12" s="20" t="inlineStr">
         <is>
           <t>Сбор ЮЛ Сингапура 2,5%</t>
         </is>
       </c>
-      <c r="T12" s="21" t="inlineStr">
+      <c r="T12" s="20" t="inlineStr">
         <is>
           <t>НПД</t>
         </is>
       </c>
-      <c r="U12" s="21" t="inlineStr">
+      <c r="U12" s="20" t="inlineStr">
         <is>
           <t>ИТОГО к оплате в месяц</t>
         </is>
       </c>
-      <c r="V12" s="22" t="inlineStr">
+      <c r="V12" s="21" t="inlineStr">
         <is>
           <t>Налог в месяц</t>
         </is>
       </c>
-      <c r="W12" s="22" t="inlineStr">
+      <c r="W12" s="21" t="inlineStr">
         <is>
           <t>Выплата ИП в месяц</t>
         </is>
       </c>
-      <c r="X12" s="23" t="inlineStr">
+      <c r="X12" s="22" t="inlineStr">
         <is>
           <t>Налог в месяц</t>
         </is>
       </c>
-      <c r="Y12" s="23" t="inlineStr">
+      <c r="Y12" s="22" t="inlineStr">
         <is>
           <t>Выплата ИП в месяц</t>
         </is>
       </c>
-      <c r="Z12" s="24" t="inlineStr">
+      <c r="Z12" s="23" t="inlineStr">
         <is>
           <t>4dev − НПД</t>
         </is>
       </c>
-      <c r="AA12" s="24" t="inlineStr">
+      <c r="AA12" s="23" t="inlineStr">
         <is>
           <t>УСН − НПД</t>
         </is>
       </c>
-      <c r="AB12" s="24" t="inlineStr">
+      <c r="AB12" s="23" t="inlineStr">
         <is>
           <t>АУСН − НПД</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="25" t="inlineStr">
-        <is>
-          <t>БВ — 15 чел.</t>
-        </is>
-      </c>
-      <c r="B13" s="26" t="n"/>
-      <c r="C13" s="26" t="n"/>
-      <c r="D13" s="26" t="n"/>
-      <c r="E13" s="26" t="n"/>
-      <c r="F13" s="26" t="n"/>
-      <c r="G13" s="26" t="n"/>
-      <c r="H13" s="26" t="n"/>
-      <c r="I13" s="26" t="n"/>
-      <c r="J13" s="26" t="n"/>
-      <c r="K13" s="26" t="n"/>
-      <c r="L13" s="26" t="n"/>
-      <c r="M13" s="26" t="n"/>
-      <c r="N13" s="26" t="n"/>
-      <c r="O13" s="26" t="n"/>
-      <c r="P13" s="26" t="n"/>
-      <c r="Q13" s="26" t="n"/>
-      <c r="R13" s="26" t="n"/>
-      <c r="S13" s="26" t="n"/>
-      <c r="T13" s="26" t="n"/>
-      <c r="U13" s="26" t="n"/>
-      <c r="V13" s="26" t="n"/>
-      <c r="W13" s="26" t="n"/>
-      <c r="X13" s="26" t="n"/>
-      <c r="Y13" s="26" t="n"/>
-      <c r="Z13" s="26" t="n"/>
-      <c r="AA13" s="26" t="n"/>
-      <c r="AB13" s="26" t="n"/>
+      <c r="A13" s="24" t="inlineStr">
+        <is>
+          <t>БВ — 16 чел.</t>
+        </is>
+      </c>
+      <c r="B13" s="25" t="n"/>
+      <c r="C13" s="25" t="n"/>
+      <c r="D13" s="25" t="n"/>
+      <c r="E13" s="25" t="n"/>
+      <c r="F13" s="25" t="n"/>
+      <c r="G13" s="25" t="n"/>
+      <c r="H13" s="25" t="n"/>
+      <c r="I13" s="25" t="n"/>
+      <c r="J13" s="25" t="n"/>
+      <c r="K13" s="25" t="n"/>
+      <c r="L13" s="25" t="n"/>
+      <c r="M13" s="25" t="n"/>
+      <c r="N13" s="25" t="n"/>
+      <c r="O13" s="25" t="n"/>
+      <c r="P13" s="25" t="n"/>
+      <c r="Q13" s="25" t="n"/>
+      <c r="R13" s="25" t="n"/>
+      <c r="S13" s="25" t="n"/>
+      <c r="T13" s="25" t="n"/>
+      <c r="U13" s="25" t="n"/>
+      <c r="V13" s="25" t="n"/>
+      <c r="W13" s="25" t="n"/>
+      <c r="X13" s="25" t="n"/>
+      <c r="Y13" s="25" t="n"/>
+      <c r="Z13" s="25" t="n"/>
+      <c r="AA13" s="25" t="n"/>
+      <c r="AB13" s="25" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="27" t="n">
+      <c r="A14" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="B14" s="28" t="inlineStr">
+      <c r="B14" s="27" t="inlineStr">
         <is>
           <t>Глубокая Яна Ярославовна</t>
         </is>
       </c>
-      <c r="C14" s="28" t="inlineStr">
+      <c r="C14" s="27" t="inlineStr">
         <is>
           <t>ТФМ (ПО)</t>
         </is>
       </c>
-      <c r="D14" s="27" t="inlineStr">
+      <c r="D14" s="26" t="inlineStr">
         <is>
           <t>БВ</t>
         </is>
       </c>
-      <c r="E14" s="27" t="inlineStr">
+      <c r="E14" s="26" t="inlineStr">
         <is>
           <t>6%</t>
         </is>
       </c>
-      <c r="F14" s="27" t="inlineStr">
+      <c r="F14" s="26" t="inlineStr">
         <is>
           <t>активен</t>
         </is>
       </c>
-      <c r="G14" s="27" t="inlineStr">
+      <c r="G14" s="26" t="inlineStr">
         <is>
           <t>2022–2026</t>
         </is>
       </c>
-      <c r="H14" s="27" t="n">
+      <c r="H14" s="26" t="n">
         <v>5</v>
       </c>
-      <c r="I14" s="29" t="n">
+      <c r="I14" s="28" t="n">
         <v>74734</v>
       </c>
-      <c r="J14" s="29" t="n">
+      <c r="J14" s="28" t="n">
         <v>1277373</v>
       </c>
-      <c r="K14" s="29" t="n">
+      <c r="K14" s="28" t="n">
         <v>2001199</v>
       </c>
       <c r="L14" s="29" t="n">
@@ -1203,7 +1208,7 @@
       <c r="K15" s="38" t="n">
         <v>1582317</v>
       </c>
-      <c r="L15" s="38" t="n">
+      <c r="L15" s="29" t="n">
         <v>1778297</v>
       </c>
       <c r="M15" s="38" t="n">
@@ -1274,55 +1279,55 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="27" t="n">
+      <c r="A16" s="26" t="n">
         <v>3</v>
       </c>
-      <c r="B16" s="28" t="inlineStr">
+      <c r="B16" s="27" t="inlineStr">
         <is>
           <t>Дроздова Мария Глебовна</t>
         </is>
       </c>
-      <c r="C16" s="28" t="inlineStr">
+      <c r="C16" s="27" t="inlineStr">
         <is>
           <t>ТФМ (ОСП)</t>
         </is>
       </c>
-      <c r="D16" s="27" t="inlineStr">
+      <c r="D16" s="26" t="inlineStr">
         <is>
           <t>БВ</t>
         </is>
       </c>
-      <c r="E16" s="27" t="inlineStr">
+      <c r="E16" s="26" t="inlineStr">
         <is>
           <t>6%</t>
         </is>
       </c>
-      <c r="F16" s="27" t="inlineStr">
+      <c r="F16" s="26" t="inlineStr">
         <is>
           <t>активен</t>
         </is>
       </c>
-      <c r="G16" s="27" t="inlineStr">
+      <c r="G16" s="26" t="inlineStr">
         <is>
           <t>2022–2026</t>
         </is>
       </c>
-      <c r="H16" s="27" t="n">
+      <c r="H16" s="26" t="n">
         <v>5</v>
       </c>
-      <c r="I16" s="29" t="n">
+      <c r="I16" s="28" t="n">
         <v>41064</v>
       </c>
-      <c r="J16" s="29" t="n">
+      <c r="J16" s="28" t="n">
         <v>637553</v>
       </c>
-      <c r="K16" s="29" t="n">
+      <c r="K16" s="28" t="n">
         <v>1442457</v>
       </c>
       <c r="L16" s="29" t="n">
         <v>1784722</v>
       </c>
-      <c r="M16" s="29" t="n">
+      <c r="M16" s="28" t="n">
         <v>1222167</v>
       </c>
       <c r="N16" s="31">
@@ -1435,8 +1440,8 @@
       <c r="K17" s="38" t="n">
         <v>1253297</v>
       </c>
-      <c r="L17" s="30" t="n">
-        <v>115745</v>
+      <c r="L17" s="29" t="n">
+        <v>1552346</v>
       </c>
       <c r="M17" s="38" t="n">
         <v>1062722</v>
@@ -1506,55 +1511,55 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="27" t="n">
+      <c r="A18" s="26" t="n">
         <v>5</v>
       </c>
-      <c r="B18" s="28" t="inlineStr">
+      <c r="B18" s="27" t="inlineStr">
         <is>
           <t>Гатиатуллина Марина Эдуардовна</t>
         </is>
       </c>
-      <c r="C18" s="28" t="inlineStr">
+      <c r="C18" s="27" t="inlineStr">
         <is>
           <t>Fansy</t>
         </is>
       </c>
-      <c r="D18" s="27" t="inlineStr">
+      <c r="D18" s="26" t="inlineStr">
         <is>
           <t>БВ</t>
         </is>
       </c>
-      <c r="E18" s="27" t="inlineStr">
+      <c r="E18" s="26" t="inlineStr">
         <is>
           <t>6%</t>
         </is>
       </c>
-      <c r="F18" s="27" t="inlineStr">
+      <c r="F18" s="26" t="inlineStr">
         <is>
           <t>активен</t>
         </is>
       </c>
-      <c r="G18" s="27" t="inlineStr">
+      <c r="G18" s="26" t="inlineStr">
         <is>
           <t>2023–2026</t>
         </is>
       </c>
-      <c r="H18" s="27" t="n">
+      <c r="H18" s="26" t="n">
         <v>4</v>
       </c>
-      <c r="I18" s="29" t="n">
+      <c r="I18" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="J18" s="29" t="n">
+      <c r="J18" s="28" t="n">
         <v>269105.17</v>
       </c>
-      <c r="K18" s="29" t="n">
+      <c r="K18" s="28" t="n">
         <v>1743298</v>
       </c>
       <c r="L18" s="29" t="n">
         <v>1991245.01</v>
       </c>
-      <c r="M18" s="29" t="n">
+      <c r="M18" s="28" t="n">
         <v>1192011.1</v>
       </c>
       <c r="N18" s="31">
@@ -1667,7 +1672,7 @@
       <c r="K19" s="30" t="n">
         <v>205851</v>
       </c>
-      <c r="L19" s="30" t="n">
+      <c r="L19" s="29" t="n">
         <v>2326991</v>
       </c>
       <c r="M19" s="38" t="n">
@@ -1738,55 +1743,55 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="27" t="n">
+      <c r="A20" s="26" t="n">
         <v>7</v>
       </c>
-      <c r="B20" s="28" t="inlineStr">
+      <c r="B20" s="27" t="inlineStr">
         <is>
           <t>Бобрышева Татьяна Сергеевна</t>
         </is>
       </c>
-      <c r="C20" s="28" t="inlineStr">
+      <c r="C20" s="27" t="inlineStr">
         <is>
           <t>ТФМ (ПО)</t>
         </is>
       </c>
-      <c r="D20" s="27" t="inlineStr">
+      <c r="D20" s="26" t="inlineStr">
         <is>
           <t>БВ</t>
         </is>
       </c>
-      <c r="E20" s="27" t="inlineStr">
+      <c r="E20" s="26" t="inlineStr">
         <is>
           <t>6%</t>
         </is>
       </c>
-      <c r="F20" s="27" t="inlineStr">
+      <c r="F20" s="26" t="inlineStr">
         <is>
           <t>активен</t>
         </is>
       </c>
-      <c r="G20" s="27" t="inlineStr">
+      <c r="G20" s="26" t="inlineStr">
         <is>
           <t>2023–2026</t>
         </is>
       </c>
-      <c r="H20" s="27" t="n">
+      <c r="H20" s="26" t="n">
         <v>4</v>
       </c>
-      <c r="I20" s="29" t="n">
+      <c r="I20" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="J20" s="29" t="n">
+      <c r="J20" s="28" t="n">
         <v>554372.52</v>
       </c>
-      <c r="K20" s="29" t="n">
+      <c r="K20" s="28" t="n">
         <v>1016796.76</v>
       </c>
-      <c r="L20" s="29" t="n">
+      <c r="L20" s="28" t="n">
         <v>1505710.52</v>
       </c>
-      <c r="M20" s="29" t="n">
+      <c r="M20" s="28" t="n">
         <v>1082430.98</v>
       </c>
       <c r="N20" s="31">
@@ -1899,7 +1904,7 @@
       <c r="K21" s="38" t="n">
         <v>690632</v>
       </c>
-      <c r="L21" s="38" t="n">
+      <c r="L21" s="29" t="n">
         <v>1072320</v>
       </c>
       <c r="M21" s="38" t="n">
@@ -1970,55 +1975,55 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="27" t="n">
+      <c r="A22" s="26" t="n">
         <v>9</v>
       </c>
-      <c r="B22" s="28" t="inlineStr">
+      <c r="B22" s="27" t="inlineStr">
         <is>
           <t>Кузнецова Светлана Дмитриевна</t>
         </is>
       </c>
-      <c r="C22" s="28" t="inlineStr">
+      <c r="C22" s="27" t="inlineStr">
         <is>
           <t>ТФМ (ПО)</t>
         </is>
       </c>
-      <c r="D22" s="27" t="inlineStr">
+      <c r="D22" s="26" t="inlineStr">
         <is>
           <t>БВ</t>
         </is>
       </c>
-      <c r="E22" s="27" t="inlineStr">
+      <c r="E22" s="26" t="inlineStr">
         <is>
           <t>6%</t>
         </is>
       </c>
-      <c r="F22" s="27" t="inlineStr">
+      <c r="F22" s="26" t="inlineStr">
         <is>
           <t>активен</t>
         </is>
       </c>
-      <c r="G22" s="27" t="inlineStr">
+      <c r="G22" s="26" t="inlineStr">
         <is>
           <t>2024–2026</t>
         </is>
       </c>
-      <c r="H22" s="27" t="n">
+      <c r="H22" s="26" t="n">
         <v>3</v>
       </c>
-      <c r="I22" s="29" t="n">
+      <c r="I22" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="J22" s="29" t="n">
+      <c r="J22" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="K22" s="29" t="n">
+      <c r="K22" s="28" t="n">
         <v>1425506.19</v>
       </c>
-      <c r="L22" s="30" t="n">
+      <c r="L22" s="29" t="n">
         <v>1685016.96</v>
       </c>
-      <c r="M22" s="29" t="n">
+      <c r="M22" s="28" t="n">
         <v>1145357.79</v>
       </c>
       <c r="N22" s="31">
@@ -2091,12 +2096,12 @@
       </c>
       <c r="B23" s="37" t="inlineStr">
         <is>
-          <t>Демакова Дарья</t>
+          <t>Тупико Олег Николаевич</t>
         </is>
       </c>
       <c r="C23" s="37" t="inlineStr">
         <is>
-          <t>ТХ</t>
+          <t>ГК (общие)</t>
         </is>
       </c>
       <c r="D23" s="36" t="inlineStr">
@@ -2128,14 +2133,14 @@
       <c r="J23" s="38" t="n">
         <v>0</v>
       </c>
-      <c r="K23" s="38" t="n">
-        <v>582823.1800000001</v>
-      </c>
-      <c r="L23" s="38" t="n">
-        <v>1530724</v>
+      <c r="K23" s="30" t="n">
+        <v>259907</v>
+      </c>
+      <c r="L23" s="29" t="n">
+        <v>2055921</v>
       </c>
       <c r="M23" s="38" t="n">
-        <v>1167329</v>
+        <v>1219304</v>
       </c>
       <c r="N23" s="39">
         <f>SUM(I23:M23)</f>
@@ -2202,56 +2207,56 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="27" t="n">
+      <c r="A24" s="26" t="n">
         <v>11</v>
       </c>
-      <c r="B24" s="28" t="inlineStr">
-        <is>
-          <t>Нуруллина Анжелика Альбертовна</t>
-        </is>
-      </c>
-      <c r="C24" s="28" t="inlineStr">
-        <is>
-          <t>Fansy</t>
-        </is>
-      </c>
-      <c r="D24" s="27" t="inlineStr">
+      <c r="B24" s="27" t="inlineStr">
+        <is>
+          <t>Демакова Дарья</t>
+        </is>
+      </c>
+      <c r="C24" s="27" t="inlineStr">
+        <is>
+          <t>ТХ</t>
+        </is>
+      </c>
+      <c r="D24" s="26" t="inlineStr">
         <is>
           <t>БВ</t>
         </is>
       </c>
-      <c r="E24" s="27" t="inlineStr">
+      <c r="E24" s="26" t="inlineStr">
         <is>
           <t>6%</t>
         </is>
       </c>
-      <c r="F24" s="27" t="inlineStr">
+      <c r="F24" s="26" t="inlineStr">
         <is>
           <t>активен</t>
         </is>
       </c>
-      <c r="G24" s="27" t="inlineStr">
+      <c r="G24" s="26" t="inlineStr">
         <is>
           <t>2024–2026</t>
         </is>
       </c>
-      <c r="H24" s="27" t="n">
+      <c r="H24" s="26" t="n">
         <v>3</v>
       </c>
-      <c r="I24" s="29" t="n">
+      <c r="I24" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="J24" s="29" t="n">
+      <c r="J24" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="K24" s="30" t="n">
-        <v>338830</v>
-      </c>
-      <c r="L24" s="30" t="n">
-        <v>1331065</v>
-      </c>
-      <c r="M24" s="29" t="n">
-        <v>741701</v>
+      <c r="K24" s="28" t="n">
+        <v>582823.1800000001</v>
+      </c>
+      <c r="L24" s="28" t="n">
+        <v>1530724</v>
+      </c>
+      <c r="M24" s="28" t="n">
+        <v>1167329</v>
       </c>
       <c r="N24" s="31">
         <f>SUM(I24:M24)</f>
@@ -2323,12 +2328,12 @@
       </c>
       <c r="B25" s="37" t="inlineStr">
         <is>
-          <t>Тупико Олег Николаевич</t>
+          <t>Нуруллина Анжелика Альбертовна</t>
         </is>
       </c>
       <c r="C25" s="37" t="inlineStr">
         <is>
-          <t>ГК (общие)</t>
+          <t>Fansy</t>
         </is>
       </c>
       <c r="D25" s="36" t="inlineStr">
@@ -2361,13 +2366,13 @@
         <v>0</v>
       </c>
       <c r="K25" s="30" t="n">
-        <v>259907</v>
-      </c>
-      <c r="L25" s="30" t="n">
-        <v>337036</v>
+        <v>338830</v>
+      </c>
+      <c r="L25" s="29" t="n">
+        <v>1468033</v>
       </c>
       <c r="M25" s="38" t="n">
-        <v>1219304</v>
+        <v>741701</v>
       </c>
       <c r="N25" s="39">
         <f>SUM(I25:M25)</f>
@@ -2434,55 +2439,55 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="27" t="n">
+      <c r="A26" s="26" t="n">
         <v>13</v>
       </c>
-      <c r="B26" s="28" t="inlineStr">
+      <c r="B26" s="27" t="inlineStr">
         <is>
           <t>Лукьянова Вера Константиновна</t>
         </is>
       </c>
-      <c r="C26" s="28" t="inlineStr">
+      <c r="C26" s="27" t="inlineStr">
         <is>
           <t>ТФМ (ПО)</t>
         </is>
       </c>
-      <c r="D26" s="27" t="inlineStr">
+      <c r="D26" s="26" t="inlineStr">
         <is>
           <t>БВ</t>
         </is>
       </c>
-      <c r="E26" s="27" t="inlineStr">
+      <c r="E26" s="26" t="inlineStr">
         <is>
           <t>6%</t>
         </is>
       </c>
-      <c r="F26" s="27" t="inlineStr">
+      <c r="F26" s="26" t="inlineStr">
         <is>
           <t>активен</t>
         </is>
       </c>
-      <c r="G26" s="27" t="inlineStr">
+      <c r="G26" s="26" t="inlineStr">
         <is>
           <t>2024–2026</t>
         </is>
       </c>
-      <c r="H26" s="27" t="n">
+      <c r="H26" s="26" t="n">
         <v>3</v>
       </c>
-      <c r="I26" s="29" t="n">
+      <c r="I26" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="J26" s="29" t="n">
+      <c r="J26" s="28" t="n">
         <v>0</v>
       </c>
       <c r="K26" s="30" t="n">
         <v>141702</v>
       </c>
-      <c r="L26" s="30" t="n">
-        <v>73617</v>
-      </c>
-      <c r="M26" s="29" t="n">
+      <c r="L26" s="29" t="n">
+        <v>1135453.68</v>
+      </c>
+      <c r="M26" s="28" t="n">
         <v>973404</v>
       </c>
       <c r="N26" s="31">
@@ -2595,8 +2600,8 @@
       <c r="K27" s="38" t="n">
         <v>0</v>
       </c>
-      <c r="L27" s="30" t="n">
-        <v>798831.01</v>
+      <c r="L27" s="29" t="n">
+        <v>1134146.01</v>
       </c>
       <c r="M27" s="38" t="n">
         <v>1362100.09</v>
@@ -2666,56 +2671,56 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="27" t="n">
+      <c r="A28" s="26" t="n">
         <v>15</v>
       </c>
-      <c r="B28" s="28" t="inlineStr">
-        <is>
-          <t>Капустина Вероника Сергеевна</t>
-        </is>
-      </c>
-      <c r="C28" s="28" t="inlineStr">
-        <is>
-          <t>ТФМ (ОСК)</t>
-        </is>
-      </c>
-      <c r="D28" s="27" t="inlineStr">
+      <c r="B28" s="27" t="inlineStr">
+        <is>
+          <t>Шультяева Елизавета Александровна</t>
+        </is>
+      </c>
+      <c r="C28" s="27" t="inlineStr">
+        <is>
+          <t>ТФМ (ПО)</t>
+        </is>
+      </c>
+      <c r="D28" s="26" t="inlineStr">
         <is>
           <t>БВ</t>
         </is>
       </c>
-      <c r="E28" s="27" t="inlineStr">
+      <c r="E28" s="26" t="inlineStr">
         <is>
           <t>6%</t>
         </is>
       </c>
-      <c r="F28" s="27" t="inlineStr">
+      <c r="F28" s="26" t="inlineStr">
         <is>
           <t>активен</t>
         </is>
       </c>
-      <c r="G28" s="27" t="inlineStr">
+      <c r="G28" s="26" t="inlineStr">
         <is>
           <t>2025–2026</t>
         </is>
       </c>
-      <c r="H28" s="27" t="n">
+      <c r="H28" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="I28" s="29" t="n">
+      <c r="I28" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="J28" s="29" t="n">
+      <c r="J28" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="K28" s="29" t="n">
+      <c r="K28" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="L28" s="29" t="n">
-        <v>214440.3</v>
-      </c>
-      <c r="M28" s="29" t="n">
-        <v>1228052.73</v>
+      <c r="L28" s="30" t="n">
+        <v>1265701.26</v>
+      </c>
+      <c r="M28" s="28" t="n">
+        <v>955013.3199999999</v>
       </c>
       <c r="N28" s="31">
         <f>SUM(I28:M28)</f>
@@ -2782,358 +2787,358 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="43" t="n"/>
-      <c r="B29" s="44" t="inlineStr">
+      <c r="A29" s="36" t="n">
+        <v>16</v>
+      </c>
+      <c r="B29" s="37" t="inlineStr">
+        <is>
+          <t>Капустина Вероника Сергеевна</t>
+        </is>
+      </c>
+      <c r="C29" s="37" t="inlineStr">
+        <is>
+          <t>ТФМ (ОСК)</t>
+        </is>
+      </c>
+      <c r="D29" s="36" t="inlineStr">
+        <is>
+          <t>БВ</t>
+        </is>
+      </c>
+      <c r="E29" s="36" t="inlineStr">
+        <is>
+          <t>6%</t>
+        </is>
+      </c>
+      <c r="F29" s="36" t="inlineStr">
+        <is>
+          <t>активен</t>
+        </is>
+      </c>
+      <c r="G29" s="36" t="inlineStr">
+        <is>
+          <t>2025–2026</t>
+        </is>
+      </c>
+      <c r="H29" s="36" t="n">
+        <v>2</v>
+      </c>
+      <c r="I29" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="J29" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="K29" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="L29" s="38" t="n">
+        <v>214440.3</v>
+      </c>
+      <c r="M29" s="38" t="n">
+        <v>1228052.73</v>
+      </c>
+      <c r="N29" s="39">
+        <f>SUM(I29:M29)</f>
+        <v/>
+      </c>
+      <c r="O29" s="39">
+        <f>M29/$C$5*(1-$AD29)</f>
+        <v/>
+      </c>
+      <c r="P29" s="40">
+        <f>IF($AD29=0,0,O29/(1-$AD29)-O29)</f>
+        <v/>
+      </c>
+      <c r="Q29" s="41">
+        <f>O29+P29</f>
+        <v/>
+      </c>
+      <c r="R29" s="40">
+        <f>O29*$C$6</f>
+        <v/>
+      </c>
+      <c r="S29" s="40">
+        <f>O29/(1-$C$7)-O29</f>
+        <v/>
+      </c>
+      <c r="T29" s="40">
+        <f>IF($AD29=0,0,O29/(1-$AD29)-O29)</f>
+        <v/>
+      </c>
+      <c r="U29" s="41">
+        <f>O29+R29+S29+T29</f>
+        <v/>
+      </c>
+      <c r="V29" s="40">
+        <f>O29/(1-$C$8)-O29</f>
+        <v/>
+      </c>
+      <c r="W29" s="41">
+        <f>O29+V29</f>
+        <v/>
+      </c>
+      <c r="X29" s="40">
+        <f>O29/(1-$C$9)-O29</f>
+        <v/>
+      </c>
+      <c r="Y29" s="41">
+        <f>O29+X29</f>
+        <v/>
+      </c>
+      <c r="Z29" s="42">
+        <f>U29-Q29</f>
+        <v/>
+      </c>
+      <c r="AA29" s="42">
+        <f>W29-Q29</f>
+        <v/>
+      </c>
+      <c r="AB29" s="42">
+        <f>Y29-Q29</f>
+        <v/>
+      </c>
+      <c r="AD29" s="35" t="n">
+        <v>0.06</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="43" t="n"/>
+      <c r="B30" s="44" t="inlineStr">
         <is>
           <t>Итого БВ</t>
         </is>
       </c>
-      <c r="C29" s="43" t="n"/>
-      <c r="D29" s="43" t="n"/>
-      <c r="E29" s="43" t="n"/>
-      <c r="F29" s="43" t="n"/>
-      <c r="G29" s="43" t="n"/>
-      <c r="H29" s="43" t="n"/>
-      <c r="I29" s="45">
-        <f>SUM(I14:I28)</f>
-        <v/>
-      </c>
-      <c r="J29" s="45">
-        <f>SUM(J14:J28)</f>
-        <v/>
-      </c>
-      <c r="K29" s="45">
-        <f>SUM(K14:K28)</f>
-        <v/>
-      </c>
-      <c r="L29" s="45">
-        <f>SUM(L14:L28)</f>
-        <v/>
-      </c>
-      <c r="M29" s="45">
-        <f>SUM(M14:M28)</f>
-        <v/>
-      </c>
-      <c r="N29" s="45">
-        <f>SUM(N14:N28)</f>
-        <v/>
-      </c>
-      <c r="O29" s="45">
-        <f>SUM(O14:O28)</f>
-        <v/>
-      </c>
-      <c r="P29" s="45">
-        <f>SUM(P14:P28)</f>
-        <v/>
-      </c>
-      <c r="Q29" s="45">
-        <f>SUM(Q14:Q28)</f>
-        <v/>
-      </c>
-      <c r="R29" s="45">
-        <f>SUM(R14:R28)</f>
-        <v/>
-      </c>
-      <c r="S29" s="45">
-        <f>SUM(S14:S28)</f>
-        <v/>
-      </c>
-      <c r="T29" s="45">
-        <f>SUM(T14:T28)</f>
-        <v/>
-      </c>
-      <c r="U29" s="45">
-        <f>SUM(U14:U28)</f>
-        <v/>
-      </c>
-      <c r="V29" s="45">
-        <f>SUM(V14:V28)</f>
-        <v/>
-      </c>
-      <c r="W29" s="45">
-        <f>SUM(W14:W28)</f>
-        <v/>
-      </c>
-      <c r="X29" s="45">
-        <f>SUM(X14:X28)</f>
-        <v/>
-      </c>
-      <c r="Y29" s="45">
-        <f>SUM(Y14:Y28)</f>
-        <v/>
-      </c>
-      <c r="Z29" s="45">
-        <f>SUM(Z14:Z28)</f>
-        <v/>
-      </c>
-      <c r="AA29" s="45">
-        <f>SUM(AA14:AA28)</f>
-        <v/>
-      </c>
-      <c r="AB29" s="45">
-        <f>SUM(AB14:AB28)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="25" t="inlineStr">
+      <c r="C30" s="43" t="n"/>
+      <c r="D30" s="43" t="n"/>
+      <c r="E30" s="43" t="n"/>
+      <c r="F30" s="43" t="n"/>
+      <c r="G30" s="43" t="n"/>
+      <c r="H30" s="43" t="n"/>
+      <c r="I30" s="45">
+        <f>SUM(I14:I29)</f>
+        <v/>
+      </c>
+      <c r="J30" s="45">
+        <f>SUM(J14:J29)</f>
+        <v/>
+      </c>
+      <c r="K30" s="45">
+        <f>SUM(K14:K29)</f>
+        <v/>
+      </c>
+      <c r="L30" s="45">
+        <f>SUM(L14:L29)</f>
+        <v/>
+      </c>
+      <c r="M30" s="45">
+        <f>SUM(M14:M29)</f>
+        <v/>
+      </c>
+      <c r="N30" s="45">
+        <f>SUM(N14:N29)</f>
+        <v/>
+      </c>
+      <c r="O30" s="45">
+        <f>SUM(O14:O29)</f>
+        <v/>
+      </c>
+      <c r="P30" s="45">
+        <f>SUM(P14:P29)</f>
+        <v/>
+      </c>
+      <c r="Q30" s="45">
+        <f>SUM(Q14:Q29)</f>
+        <v/>
+      </c>
+      <c r="R30" s="45">
+        <f>SUM(R14:R29)</f>
+        <v/>
+      </c>
+      <c r="S30" s="45">
+        <f>SUM(S14:S29)</f>
+        <v/>
+      </c>
+      <c r="T30" s="45">
+        <f>SUM(T14:T29)</f>
+        <v/>
+      </c>
+      <c r="U30" s="45">
+        <f>SUM(U14:U29)</f>
+        <v/>
+      </c>
+      <c r="V30" s="45">
+        <f>SUM(V14:V29)</f>
+        <v/>
+      </c>
+      <c r="W30" s="45">
+        <f>SUM(W14:W29)</f>
+        <v/>
+      </c>
+      <c r="X30" s="45">
+        <f>SUM(X14:X29)</f>
+        <v/>
+      </c>
+      <c r="Y30" s="45">
+        <f>SUM(Y14:Y29)</f>
+        <v/>
+      </c>
+      <c r="Z30" s="45">
+        <f>SUM(Z14:Z29)</f>
+        <v/>
+      </c>
+      <c r="AA30" s="45">
+        <f>SUM(AA14:AA29)</f>
+        <v/>
+      </c>
+      <c r="AB30" s="45">
+        <f>SUM(AB14:AB29)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="24" t="inlineStr">
         <is>
           <t>АС — 4 чел.</t>
         </is>
       </c>
-      <c r="B31" s="26" t="n"/>
-      <c r="C31" s="26" t="n"/>
-      <c r="D31" s="26" t="n"/>
-      <c r="E31" s="26" t="n"/>
-      <c r="F31" s="26" t="n"/>
-      <c r="G31" s="26" t="n"/>
-      <c r="H31" s="26" t="n"/>
-      <c r="I31" s="26" t="n"/>
-      <c r="J31" s="26" t="n"/>
-      <c r="K31" s="26" t="n"/>
-      <c r="L31" s="26" t="n"/>
-      <c r="M31" s="26" t="n"/>
-      <c r="N31" s="26" t="n"/>
-      <c r="O31" s="26" t="n"/>
-      <c r="P31" s="26" t="n"/>
-      <c r="Q31" s="26" t="n"/>
-      <c r="R31" s="26" t="n"/>
-      <c r="S31" s="26" t="n"/>
-      <c r="T31" s="26" t="n"/>
-      <c r="U31" s="26" t="n"/>
-      <c r="V31" s="26" t="n"/>
-      <c r="W31" s="26" t="n"/>
-      <c r="X31" s="26" t="n"/>
-      <c r="Y31" s="26" t="n"/>
-      <c r="Z31" s="26" t="n"/>
-      <c r="AA31" s="26" t="n"/>
-      <c r="AB31" s="26" t="n"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="27" t="n">
-        <v>16</v>
-      </c>
-      <c r="B32" s="28" t="inlineStr">
+      <c r="B32" s="25" t="n"/>
+      <c r="C32" s="25" t="n"/>
+      <c r="D32" s="25" t="n"/>
+      <c r="E32" s="25" t="n"/>
+      <c r="F32" s="25" t="n"/>
+      <c r="G32" s="25" t="n"/>
+      <c r="H32" s="25" t="n"/>
+      <c r="I32" s="25" t="n"/>
+      <c r="J32" s="25" t="n"/>
+      <c r="K32" s="25" t="n"/>
+      <c r="L32" s="25" t="n"/>
+      <c r="M32" s="25" t="n"/>
+      <c r="N32" s="25" t="n"/>
+      <c r="O32" s="25" t="n"/>
+      <c r="P32" s="25" t="n"/>
+      <c r="Q32" s="25" t="n"/>
+      <c r="R32" s="25" t="n"/>
+      <c r="S32" s="25" t="n"/>
+      <c r="T32" s="25" t="n"/>
+      <c r="U32" s="25" t="n"/>
+      <c r="V32" s="25" t="n"/>
+      <c r="W32" s="25" t="n"/>
+      <c r="X32" s="25" t="n"/>
+      <c r="Y32" s="25" t="n"/>
+      <c r="Z32" s="25" t="n"/>
+      <c r="AA32" s="25" t="n"/>
+      <c r="AB32" s="25" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="26" t="n">
+        <v>17</v>
+      </c>
+      <c r="B33" s="27" t="inlineStr">
         <is>
           <t>Грудинин Алексей Сергеевич</t>
         </is>
       </c>
-      <c r="C32" s="28" t="inlineStr">
+      <c r="C33" s="27" t="inlineStr">
         <is>
           <t>ТФМ (ПО)</t>
         </is>
       </c>
-      <c r="D32" s="27" t="inlineStr">
+      <c r="D33" s="26" t="inlineStr">
         <is>
           <t>АС</t>
         </is>
       </c>
-      <c r="E32" s="27" t="inlineStr">
+      <c r="E33" s="26" t="inlineStr">
         <is>
           <t>6%</t>
         </is>
       </c>
-      <c r="F32" s="27" t="inlineStr">
+      <c r="F33" s="26" t="inlineStr">
         <is>
           <t>активен</t>
         </is>
       </c>
-      <c r="G32" s="27" t="inlineStr">
+      <c r="G33" s="26" t="inlineStr">
         <is>
           <t>2022–2026</t>
         </is>
       </c>
-      <c r="H32" s="27" t="n">
+      <c r="H33" s="26" t="n">
         <v>5</v>
       </c>
-      <c r="I32" s="29" t="n">
+      <c r="I33" s="28" t="n">
         <v>267577.88</v>
       </c>
-      <c r="J32" s="29" t="n">
+      <c r="J33" s="28" t="n">
         <v>960405.97</v>
       </c>
-      <c r="K32" s="29" t="n">
+      <c r="K33" s="28" t="n">
         <v>1372957.36</v>
       </c>
-      <c r="L32" s="29" t="n">
+      <c r="L33" s="28" t="n">
         <v>1558585.08</v>
       </c>
-      <c r="M32" s="29" t="n">
+      <c r="M33" s="28" t="n">
         <v>938053.12</v>
       </c>
-      <c r="N32" s="31">
-        <f>SUM(I32:M32)</f>
-        <v/>
-      </c>
-      <c r="O32" s="31">
-        <f>M32/$C$5*(1-$AD32)</f>
-        <v/>
-      </c>
-      <c r="P32" s="32">
-        <f>IF($AD32=0,0,O32/(1-$AD32)-O32)</f>
-        <v/>
-      </c>
-      <c r="Q32" s="33">
-        <f>O32+P32</f>
-        <v/>
-      </c>
-      <c r="R32" s="32">
-        <f>O32*$C$6</f>
-        <v/>
-      </c>
-      <c r="S32" s="32">
-        <f>O32/(1-$C$7)-O32</f>
-        <v/>
-      </c>
-      <c r="T32" s="32">
-        <f>IF($AD32=0,0,O32/(1-$AD32)-O32)</f>
-        <v/>
-      </c>
-      <c r="U32" s="33">
-        <f>O32+R32+S32+T32</f>
-        <v/>
-      </c>
-      <c r="V32" s="32">
-        <f>O32/(1-$C$8)-O32</f>
-        <v/>
-      </c>
-      <c r="W32" s="33">
-        <f>O32+V32</f>
-        <v/>
-      </c>
-      <c r="X32" s="32">
-        <f>O32/(1-$C$9)-O32</f>
-        <v/>
-      </c>
-      <c r="Y32" s="33">
-        <f>O32+X32</f>
-        <v/>
-      </c>
-      <c r="Z32" s="34">
-        <f>U32-Q32</f>
-        <v/>
-      </c>
-      <c r="AA32" s="34">
-        <f>W32-Q32</f>
-        <v/>
-      </c>
-      <c r="AB32" s="34">
-        <f>Y32-Q32</f>
-        <v/>
-      </c>
-      <c r="AD32" s="35" t="n">
-        <v>0.06</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="36" t="n">
-        <v>17</v>
-      </c>
-      <c r="B33" s="37" t="inlineStr">
-        <is>
-          <t>Репетенко Инна Эдуардовна</t>
-        </is>
-      </c>
-      <c r="C33" s="37" t="inlineStr">
-        <is>
-          <t>ТФМ (ОРБ)</t>
-        </is>
-      </c>
-      <c r="D33" s="36" t="inlineStr">
-        <is>
-          <t>АС</t>
-        </is>
-      </c>
-      <c r="E33" s="36" t="inlineStr">
-        <is>
-          <t>6%</t>
-        </is>
-      </c>
-      <c r="F33" s="36" t="inlineStr">
-        <is>
-          <t>активен</t>
-        </is>
-      </c>
-      <c r="G33" s="36" t="inlineStr">
-        <is>
-          <t>2022–2026</t>
-        </is>
-      </c>
-      <c r="H33" s="36" t="n">
-        <v>5</v>
-      </c>
-      <c r="I33" s="30" t="n">
-        <v>112190</v>
-      </c>
-      <c r="J33" s="30" t="n">
-        <v>246600</v>
-      </c>
-      <c r="K33" s="30" t="n">
-        <v>415655.93</v>
-      </c>
-      <c r="L33" s="30" t="n">
-        <v>142973.52</v>
-      </c>
-      <c r="M33" s="38" t="n">
-        <v>905821.35</v>
-      </c>
-      <c r="N33" s="39">
+      <c r="N33" s="31">
         <f>SUM(I33:M33)</f>
         <v/>
       </c>
-      <c r="O33" s="39">
+      <c r="O33" s="31">
         <f>M33/$C$5*(1-$AD33)</f>
         <v/>
       </c>
-      <c r="P33" s="40">
+      <c r="P33" s="32">
         <f>IF($AD33=0,0,O33/(1-$AD33)-O33)</f>
         <v/>
       </c>
-      <c r="Q33" s="41">
+      <c r="Q33" s="33">
         <f>O33+P33</f>
         <v/>
       </c>
-      <c r="R33" s="40">
+      <c r="R33" s="32">
         <f>O33*$C$6</f>
         <v/>
       </c>
-      <c r="S33" s="40">
+      <c r="S33" s="32">
         <f>O33/(1-$C$7)-O33</f>
         <v/>
       </c>
-      <c r="T33" s="40">
+      <c r="T33" s="32">
         <f>IF($AD33=0,0,O33/(1-$AD33)-O33)</f>
         <v/>
       </c>
-      <c r="U33" s="41">
+      <c r="U33" s="33">
         <f>O33+R33+S33+T33</f>
         <v/>
       </c>
-      <c r="V33" s="40">
+      <c r="V33" s="32">
         <f>O33/(1-$C$8)-O33</f>
         <v/>
       </c>
-      <c r="W33" s="41">
+      <c r="W33" s="33">
         <f>O33+V33</f>
         <v/>
       </c>
-      <c r="X33" s="40">
+      <c r="X33" s="32">
         <f>O33/(1-$C$9)-O33</f>
         <v/>
       </c>
-      <c r="Y33" s="41">
+      <c r="Y33" s="33">
         <f>O33+X33</f>
         <v/>
       </c>
-      <c r="Z33" s="42">
+      <c r="Z33" s="34">
         <f>U33-Q33</f>
         <v/>
       </c>
-      <c r="AA33" s="42">
+      <c r="AA33" s="34">
         <f>W33-Q33</f>
         <v/>
       </c>
-      <c r="AB33" s="42">
+      <c r="AB33" s="34">
         <f>Y33-Q33</f>
         <v/>
       </c>
@@ -3142,114 +3147,114 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="27" t="n">
+      <c r="A34" s="36" t="n">
         <v>18</v>
       </c>
-      <c r="B34" s="28" t="inlineStr">
-        <is>
-          <t>Жиркова Валентина Александровна</t>
-        </is>
-      </c>
-      <c r="C34" s="28" t="inlineStr">
-        <is>
-          <t>ТФМ (ПО)</t>
-        </is>
-      </c>
-      <c r="D34" s="27" t="inlineStr">
+      <c r="B34" s="37" t="inlineStr">
+        <is>
+          <t>Репетенко Инна Эдуардовна</t>
+        </is>
+      </c>
+      <c r="C34" s="37" t="inlineStr">
+        <is>
+          <t>ТФМ (ОРБ)</t>
+        </is>
+      </c>
+      <c r="D34" s="36" t="inlineStr">
         <is>
           <t>АС</t>
         </is>
       </c>
-      <c r="E34" s="27" t="inlineStr">
+      <c r="E34" s="36" t="inlineStr">
         <is>
           <t>6%</t>
         </is>
       </c>
-      <c r="F34" s="27" t="inlineStr">
+      <c r="F34" s="36" t="inlineStr">
         <is>
           <t>активен</t>
         </is>
       </c>
-      <c r="G34" s="27" t="inlineStr">
-        <is>
-          <t>2023–2026</t>
-        </is>
-      </c>
-      <c r="H34" s="27" t="n">
-        <v>4</v>
-      </c>
-      <c r="I34" s="29" t="n">
-        <v>0</v>
-      </c>
-      <c r="J34" s="29" t="n">
-        <v>257222.24</v>
-      </c>
-      <c r="K34" s="29" t="n">
-        <v>1497661</v>
+      <c r="G34" s="36" t="inlineStr">
+        <is>
+          <t>2022–2026</t>
+        </is>
+      </c>
+      <c r="H34" s="36" t="n">
+        <v>5</v>
+      </c>
+      <c r="I34" s="30" t="n">
+        <v>112190</v>
+      </c>
+      <c r="J34" s="30" t="n">
+        <v>246600</v>
+      </c>
+      <c r="K34" s="30" t="n">
+        <v>415655.93</v>
       </c>
       <c r="L34" s="29" t="n">
-        <v>2201639.5</v>
-      </c>
-      <c r="M34" s="30" t="n">
-        <v>1656517.19</v>
-      </c>
-      <c r="N34" s="31">
+        <v>1639825.6</v>
+      </c>
+      <c r="M34" s="38" t="n">
+        <v>905821.35</v>
+      </c>
+      <c r="N34" s="39">
         <f>SUM(I34:M34)</f>
         <v/>
       </c>
-      <c r="O34" s="31">
+      <c r="O34" s="39">
         <f>M34/$C$5*(1-$AD34)</f>
         <v/>
       </c>
-      <c r="P34" s="32">
+      <c r="P34" s="40">
         <f>IF($AD34=0,0,O34/(1-$AD34)-O34)</f>
         <v/>
       </c>
-      <c r="Q34" s="33">
+      <c r="Q34" s="41">
         <f>O34+P34</f>
         <v/>
       </c>
-      <c r="R34" s="32">
+      <c r="R34" s="40">
         <f>O34*$C$6</f>
         <v/>
       </c>
-      <c r="S34" s="32">
+      <c r="S34" s="40">
         <f>O34/(1-$C$7)-O34</f>
         <v/>
       </c>
-      <c r="T34" s="32">
+      <c r="T34" s="40">
         <f>IF($AD34=0,0,O34/(1-$AD34)-O34)</f>
         <v/>
       </c>
-      <c r="U34" s="33">
+      <c r="U34" s="41">
         <f>O34+R34+S34+T34</f>
         <v/>
       </c>
-      <c r="V34" s="32">
+      <c r="V34" s="40">
         <f>O34/(1-$C$8)-O34</f>
         <v/>
       </c>
-      <c r="W34" s="33">
+      <c r="W34" s="41">
         <f>O34+V34</f>
         <v/>
       </c>
-      <c r="X34" s="32">
+      <c r="X34" s="40">
         <f>O34/(1-$C$9)-O34</f>
         <v/>
       </c>
-      <c r="Y34" s="33">
+      <c r="Y34" s="41">
         <f>O34+X34</f>
         <v/>
       </c>
-      <c r="Z34" s="34">
+      <c r="Z34" s="42">
         <f>U34-Q34</f>
         <v/>
       </c>
-      <c r="AA34" s="34">
+      <c r="AA34" s="42">
         <f>W34-Q34</f>
         <v/>
       </c>
-      <c r="AB34" s="34">
+      <c r="AB34" s="42">
         <f>Y34-Q34</f>
         <v/>
       </c>
@@ -3258,114 +3263,114 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="36" t="n">
+      <c r="A35" s="26" t="n">
         <v>19</v>
       </c>
-      <c r="B35" s="37" t="inlineStr">
-        <is>
-          <t>Возмищева Ксения Дмитриевна</t>
-        </is>
-      </c>
-      <c r="C35" s="37" t="inlineStr">
-        <is>
-          <t>ТФМ (ОРБ)</t>
-        </is>
-      </c>
-      <c r="D35" s="36" t="inlineStr">
+      <c r="B35" s="27" t="inlineStr">
+        <is>
+          <t>Жиркова Валентина Александровна</t>
+        </is>
+      </c>
+      <c r="C35" s="27" t="inlineStr">
+        <is>
+          <t>ТФМ (ПО)</t>
+        </is>
+      </c>
+      <c r="D35" s="26" t="inlineStr">
         <is>
           <t>АС</t>
         </is>
       </c>
-      <c r="E35" s="36" t="inlineStr">
+      <c r="E35" s="26" t="inlineStr">
         <is>
           <t>6%</t>
         </is>
       </c>
-      <c r="F35" s="36" t="inlineStr">
+      <c r="F35" s="26" t="inlineStr">
         <is>
           <t>активен</t>
         </is>
       </c>
-      <c r="G35" s="36" t="inlineStr">
-        <is>
-          <t>2024–2026</t>
-        </is>
-      </c>
-      <c r="H35" s="36" t="n">
-        <v>3</v>
-      </c>
-      <c r="I35" s="38" t="n">
+      <c r="G35" s="26" t="inlineStr">
+        <is>
+          <t>2023–2026</t>
+        </is>
+      </c>
+      <c r="H35" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="I35" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="J35" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="K35" s="38" t="n">
-        <v>333311.66</v>
-      </c>
-      <c r="L35" s="38" t="n">
-        <v>1347175.74</v>
-      </c>
-      <c r="M35" s="38" t="n">
-        <v>1267879.25</v>
-      </c>
-      <c r="N35" s="39">
+      <c r="J35" s="28" t="n">
+        <v>257222.24</v>
+      </c>
+      <c r="K35" s="28" t="n">
+        <v>1497661</v>
+      </c>
+      <c r="L35" s="29" t="n">
+        <v>2201639.5</v>
+      </c>
+      <c r="M35" s="30" t="n">
+        <v>1656517.19</v>
+      </c>
+      <c r="N35" s="31">
         <f>SUM(I35:M35)</f>
         <v/>
       </c>
-      <c r="O35" s="39">
+      <c r="O35" s="31">
         <f>M35/$C$5*(1-$AD35)</f>
         <v/>
       </c>
-      <c r="P35" s="40">
+      <c r="P35" s="32">
         <f>IF($AD35=0,0,O35/(1-$AD35)-O35)</f>
         <v/>
       </c>
-      <c r="Q35" s="41">
+      <c r="Q35" s="33">
         <f>O35+P35</f>
         <v/>
       </c>
-      <c r="R35" s="40">
+      <c r="R35" s="32">
         <f>O35*$C$6</f>
         <v/>
       </c>
-      <c r="S35" s="40">
+      <c r="S35" s="32">
         <f>O35/(1-$C$7)-O35</f>
         <v/>
       </c>
-      <c r="T35" s="40">
+      <c r="T35" s="32">
         <f>IF($AD35=0,0,O35/(1-$AD35)-O35)</f>
         <v/>
       </c>
-      <c r="U35" s="41">
+      <c r="U35" s="33">
         <f>O35+R35+S35+T35</f>
         <v/>
       </c>
-      <c r="V35" s="40">
+      <c r="V35" s="32">
         <f>O35/(1-$C$8)-O35</f>
         <v/>
       </c>
-      <c r="W35" s="41">
+      <c r="W35" s="33">
         <f>O35+V35</f>
         <v/>
       </c>
-      <c r="X35" s="40">
+      <c r="X35" s="32">
         <f>O35/(1-$C$9)-O35</f>
         <v/>
       </c>
-      <c r="Y35" s="41">
+      <c r="Y35" s="33">
         <f>O35+X35</f>
         <v/>
       </c>
-      <c r="Z35" s="42">
+      <c r="Z35" s="34">
         <f>U35-Q35</f>
         <v/>
       </c>
-      <c r="AA35" s="42">
+      <c r="AA35" s="34">
         <f>W35-Q35</f>
         <v/>
       </c>
-      <c r="AB35" s="42">
+      <c r="AB35" s="34">
         <f>Y35-Q35</f>
         <v/>
       </c>
@@ -3374,815 +3379,945 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="43" t="n"/>
-      <c r="B36" s="44" t="inlineStr">
+      <c r="A36" s="36" t="n">
+        <v>20</v>
+      </c>
+      <c r="B36" s="37" t="inlineStr">
+        <is>
+          <t>Возмищева Ксения Дмитриевна</t>
+        </is>
+      </c>
+      <c r="C36" s="37" t="inlineStr">
+        <is>
+          <t>ТФМ (ОРБ)</t>
+        </is>
+      </c>
+      <c r="D36" s="36" t="inlineStr">
+        <is>
+          <t>АС</t>
+        </is>
+      </c>
+      <c r="E36" s="36" t="inlineStr">
+        <is>
+          <t>6%</t>
+        </is>
+      </c>
+      <c r="F36" s="36" t="inlineStr">
+        <is>
+          <t>активен</t>
+        </is>
+      </c>
+      <c r="G36" s="36" t="inlineStr">
+        <is>
+          <t>2024–2026</t>
+        </is>
+      </c>
+      <c r="H36" s="36" t="n">
+        <v>3</v>
+      </c>
+      <c r="I36" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="J36" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="K36" s="38" t="n">
+        <v>333311.66</v>
+      </c>
+      <c r="L36" s="38" t="n">
+        <v>1347175.74</v>
+      </c>
+      <c r="M36" s="38" t="n">
+        <v>1267879.25</v>
+      </c>
+      <c r="N36" s="39">
+        <f>SUM(I36:M36)</f>
+        <v/>
+      </c>
+      <c r="O36" s="39">
+        <f>M36/$C$5*(1-$AD36)</f>
+        <v/>
+      </c>
+      <c r="P36" s="40">
+        <f>IF($AD36=0,0,O36/(1-$AD36)-O36)</f>
+        <v/>
+      </c>
+      <c r="Q36" s="41">
+        <f>O36+P36</f>
+        <v/>
+      </c>
+      <c r="R36" s="40">
+        <f>O36*$C$6</f>
+        <v/>
+      </c>
+      <c r="S36" s="40">
+        <f>O36/(1-$C$7)-O36</f>
+        <v/>
+      </c>
+      <c r="T36" s="40">
+        <f>IF($AD36=0,0,O36/(1-$AD36)-O36)</f>
+        <v/>
+      </c>
+      <c r="U36" s="41">
+        <f>O36+R36+S36+T36</f>
+        <v/>
+      </c>
+      <c r="V36" s="40">
+        <f>O36/(1-$C$8)-O36</f>
+        <v/>
+      </c>
+      <c r="W36" s="41">
+        <f>O36+V36</f>
+        <v/>
+      </c>
+      <c r="X36" s="40">
+        <f>O36/(1-$C$9)-O36</f>
+        <v/>
+      </c>
+      <c r="Y36" s="41">
+        <f>O36+X36</f>
+        <v/>
+      </c>
+      <c r="Z36" s="42">
+        <f>U36-Q36</f>
+        <v/>
+      </c>
+      <c r="AA36" s="42">
+        <f>W36-Q36</f>
+        <v/>
+      </c>
+      <c r="AB36" s="42">
+        <f>Y36-Q36</f>
+        <v/>
+      </c>
+      <c r="AD36" s="35" t="n">
+        <v>0.06</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="43" t="n"/>
+      <c r="B37" s="44" t="inlineStr">
         <is>
           <t>Итого АС</t>
         </is>
       </c>
-      <c r="C36" s="43" t="n"/>
-      <c r="D36" s="43" t="n"/>
-      <c r="E36" s="43" t="n"/>
-      <c r="F36" s="43" t="n"/>
-      <c r="G36" s="43" t="n"/>
-      <c r="H36" s="43" t="n"/>
-      <c r="I36" s="45">
-        <f>SUM(I32:I35)</f>
-        <v/>
-      </c>
-      <c r="J36" s="45">
-        <f>SUM(J32:J35)</f>
-        <v/>
-      </c>
-      <c r="K36" s="45">
-        <f>SUM(K32:K35)</f>
-        <v/>
-      </c>
-      <c r="L36" s="45">
-        <f>SUM(L32:L35)</f>
-        <v/>
-      </c>
-      <c r="M36" s="45">
-        <f>SUM(M32:M35)</f>
-        <v/>
-      </c>
-      <c r="N36" s="45">
-        <f>SUM(N32:N35)</f>
-        <v/>
-      </c>
-      <c r="O36" s="45">
-        <f>SUM(O32:O35)</f>
-        <v/>
-      </c>
-      <c r="P36" s="45">
-        <f>SUM(P32:P35)</f>
-        <v/>
-      </c>
-      <c r="Q36" s="45">
-        <f>SUM(Q32:Q35)</f>
-        <v/>
-      </c>
-      <c r="R36" s="45">
-        <f>SUM(R32:R35)</f>
-        <v/>
-      </c>
-      <c r="S36" s="45">
-        <f>SUM(S32:S35)</f>
-        <v/>
-      </c>
-      <c r="T36" s="45">
-        <f>SUM(T32:T35)</f>
-        <v/>
-      </c>
-      <c r="U36" s="45">
-        <f>SUM(U32:U35)</f>
-        <v/>
-      </c>
-      <c r="V36" s="45">
-        <f>SUM(V32:V35)</f>
-        <v/>
-      </c>
-      <c r="W36" s="45">
-        <f>SUM(W32:W35)</f>
-        <v/>
-      </c>
-      <c r="X36" s="45">
-        <f>SUM(X32:X35)</f>
-        <v/>
-      </c>
-      <c r="Y36" s="45">
-        <f>SUM(Y32:Y35)</f>
-        <v/>
-      </c>
-      <c r="Z36" s="45">
-        <f>SUM(Z32:Z35)</f>
-        <v/>
-      </c>
-      <c r="AA36" s="45">
-        <f>SUM(AA32:AA35)</f>
-        <v/>
-      </c>
-      <c r="AB36" s="45">
-        <f>SUM(AB32:AB35)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="25" t="inlineStr">
+      <c r="C37" s="43" t="n"/>
+      <c r="D37" s="43" t="n"/>
+      <c r="E37" s="43" t="n"/>
+      <c r="F37" s="43" t="n"/>
+      <c r="G37" s="43" t="n"/>
+      <c r="H37" s="43" t="n"/>
+      <c r="I37" s="45">
+        <f>SUM(I33:I36)</f>
+        <v/>
+      </c>
+      <c r="J37" s="45">
+        <f>SUM(J33:J36)</f>
+        <v/>
+      </c>
+      <c r="K37" s="45">
+        <f>SUM(K33:K36)</f>
+        <v/>
+      </c>
+      <c r="L37" s="45">
+        <f>SUM(L33:L36)</f>
+        <v/>
+      </c>
+      <c r="M37" s="45">
+        <f>SUM(M33:M36)</f>
+        <v/>
+      </c>
+      <c r="N37" s="45">
+        <f>SUM(N33:N36)</f>
+        <v/>
+      </c>
+      <c r="O37" s="45">
+        <f>SUM(O33:O36)</f>
+        <v/>
+      </c>
+      <c r="P37" s="45">
+        <f>SUM(P33:P36)</f>
+        <v/>
+      </c>
+      <c r="Q37" s="45">
+        <f>SUM(Q33:Q36)</f>
+        <v/>
+      </c>
+      <c r="R37" s="45">
+        <f>SUM(R33:R36)</f>
+        <v/>
+      </c>
+      <c r="S37" s="45">
+        <f>SUM(S33:S36)</f>
+        <v/>
+      </c>
+      <c r="T37" s="45">
+        <f>SUM(T33:T36)</f>
+        <v/>
+      </c>
+      <c r="U37" s="45">
+        <f>SUM(U33:U36)</f>
+        <v/>
+      </c>
+      <c r="V37" s="45">
+        <f>SUM(V33:V36)</f>
+        <v/>
+      </c>
+      <c r="W37" s="45">
+        <f>SUM(W33:W36)</f>
+        <v/>
+      </c>
+      <c r="X37" s="45">
+        <f>SUM(X33:X36)</f>
+        <v/>
+      </c>
+      <c r="Y37" s="45">
+        <f>SUM(Y33:Y36)</f>
+        <v/>
+      </c>
+      <c r="Z37" s="45">
+        <f>SUM(Z33:Z36)</f>
+        <v/>
+      </c>
+      <c r="AA37" s="45">
+        <f>SUM(AA33:AA36)</f>
+        <v/>
+      </c>
+      <c r="AB37" s="45">
+        <f>SUM(AB33:AB36)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="24" t="inlineStr">
         <is>
           <t>ИП МТ — 1 чел.</t>
         </is>
       </c>
-      <c r="B38" s="26" t="n"/>
-      <c r="C38" s="26" t="n"/>
-      <c r="D38" s="26" t="n"/>
-      <c r="E38" s="26" t="n"/>
-      <c r="F38" s="26" t="n"/>
-      <c r="G38" s="26" t="n"/>
-      <c r="H38" s="26" t="n"/>
-      <c r="I38" s="26" t="n"/>
-      <c r="J38" s="26" t="n"/>
-      <c r="K38" s="26" t="n"/>
-      <c r="L38" s="26" t="n"/>
-      <c r="M38" s="26" t="n"/>
-      <c r="N38" s="26" t="n"/>
-      <c r="O38" s="26" t="n"/>
-      <c r="P38" s="26" t="n"/>
-      <c r="Q38" s="26" t="n"/>
-      <c r="R38" s="26" t="n"/>
-      <c r="S38" s="26" t="n"/>
-      <c r="T38" s="26" t="n"/>
-      <c r="U38" s="26" t="n"/>
-      <c r="V38" s="26" t="n"/>
-      <c r="W38" s="26" t="n"/>
-      <c r="X38" s="26" t="n"/>
-      <c r="Y38" s="26" t="n"/>
-      <c r="Z38" s="26" t="n"/>
-      <c r="AA38" s="26" t="n"/>
-      <c r="AB38" s="26" t="n"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="27" t="n">
-        <v>20</v>
-      </c>
-      <c r="B39" s="28" t="inlineStr">
+      <c r="B39" s="25" t="n"/>
+      <c r="C39" s="25" t="n"/>
+      <c r="D39" s="25" t="n"/>
+      <c r="E39" s="25" t="n"/>
+      <c r="F39" s="25" t="n"/>
+      <c r="G39" s="25" t="n"/>
+      <c r="H39" s="25" t="n"/>
+      <c r="I39" s="25" t="n"/>
+      <c r="J39" s="25" t="n"/>
+      <c r="K39" s="25" t="n"/>
+      <c r="L39" s="25" t="n"/>
+      <c r="M39" s="25" t="n"/>
+      <c r="N39" s="25" t="n"/>
+      <c r="O39" s="25" t="n"/>
+      <c r="P39" s="25" t="n"/>
+      <c r="Q39" s="25" t="n"/>
+      <c r="R39" s="25" t="n"/>
+      <c r="S39" s="25" t="n"/>
+      <c r="T39" s="25" t="n"/>
+      <c r="U39" s="25" t="n"/>
+      <c r="V39" s="25" t="n"/>
+      <c r="W39" s="25" t="n"/>
+      <c r="X39" s="25" t="n"/>
+      <c r="Y39" s="25" t="n"/>
+      <c r="Z39" s="25" t="n"/>
+      <c r="AA39" s="25" t="n"/>
+      <c r="AB39" s="25" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="26" t="n">
+        <v>21</v>
+      </c>
+      <c r="B40" s="27" t="inlineStr">
         <is>
           <t>Злобин Николай Алексеевич</t>
         </is>
       </c>
-      <c r="C39" s="28" t="inlineStr">
+      <c r="C40" s="27" t="inlineStr">
         <is>
           <t>Fansy</t>
         </is>
       </c>
-      <c r="D39" s="27" t="inlineStr">
+      <c r="D40" s="26" t="inlineStr">
         <is>
           <t>ИП МТ</t>
         </is>
       </c>
-      <c r="E39" s="27" t="inlineStr">
+      <c r="E40" s="26" t="inlineStr">
         <is>
           <t>6%</t>
         </is>
       </c>
-      <c r="F39" s="27" t="inlineStr">
+      <c r="F40" s="26" t="inlineStr">
         <is>
           <t>активен</t>
         </is>
       </c>
-      <c r="G39" s="27" t="inlineStr">
+      <c r="G40" s="26" t="inlineStr">
         <is>
           <t>2023–2026</t>
         </is>
       </c>
-      <c r="H39" s="27" t="n">
+      <c r="H40" s="26" t="n">
         <v>4</v>
       </c>
-      <c r="I39" s="29" t="n">
+      <c r="I40" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="J39" s="29" t="n">
+      <c r="J40" s="28" t="n">
         <v>231383</v>
       </c>
-      <c r="K39" s="29" t="n">
+      <c r="K40" s="28" t="n">
         <v>2343163.34</v>
       </c>
-      <c r="L39" s="29" t="n">
+      <c r="L40" s="28" t="n">
         <v>2601170</v>
       </c>
-      <c r="M39" s="29" t="n">
+      <c r="M40" s="28" t="n">
         <v>1832861.81</v>
       </c>
-      <c r="N39" s="31">
-        <f>SUM(I39:M39)</f>
-        <v/>
-      </c>
-      <c r="O39" s="31">
-        <f>M39/$C$5*(1-$AD39)</f>
-        <v/>
-      </c>
-      <c r="P39" s="32">
-        <f>IF($AD39=0,0,O39/(1-$AD39)-O39)</f>
-        <v/>
-      </c>
-      <c r="Q39" s="33">
-        <f>O39+P39</f>
-        <v/>
-      </c>
-      <c r="R39" s="32">
-        <f>O39*$C$6</f>
-        <v/>
-      </c>
-      <c r="S39" s="32">
-        <f>O39/(1-$C$7)-O39</f>
-        <v/>
-      </c>
-      <c r="T39" s="32">
-        <f>IF($AD39=0,0,O39/(1-$AD39)-O39)</f>
-        <v/>
-      </c>
-      <c r="U39" s="33">
-        <f>O39+R39+S39+T39</f>
-        <v/>
-      </c>
-      <c r="V39" s="32">
-        <f>O39/(1-$C$8)-O39</f>
-        <v/>
-      </c>
-      <c r="W39" s="33">
-        <f>O39+V39</f>
-        <v/>
-      </c>
-      <c r="X39" s="32">
-        <f>O39/(1-$C$9)-O39</f>
-        <v/>
-      </c>
-      <c r="Y39" s="33">
-        <f>O39+X39</f>
-        <v/>
-      </c>
-      <c r="Z39" s="34">
-        <f>U39-Q39</f>
-        <v/>
-      </c>
-      <c r="AA39" s="34">
-        <f>W39-Q39</f>
-        <v/>
-      </c>
-      <c r="AB39" s="34">
-        <f>Y39-Q39</f>
-        <v/>
-      </c>
-      <c r="AD39" s="35" t="n">
+      <c r="N40" s="31">
+        <f>SUM(I40:M40)</f>
+        <v/>
+      </c>
+      <c r="O40" s="31">
+        <f>M40/$C$5*(1-$AD40)</f>
+        <v/>
+      </c>
+      <c r="P40" s="32">
+        <f>IF($AD40=0,0,O40/(1-$AD40)-O40)</f>
+        <v/>
+      </c>
+      <c r="Q40" s="33">
+        <f>O40+P40</f>
+        <v/>
+      </c>
+      <c r="R40" s="32">
+        <f>O40*$C$6</f>
+        <v/>
+      </c>
+      <c r="S40" s="32">
+        <f>O40/(1-$C$7)-O40</f>
+        <v/>
+      </c>
+      <c r="T40" s="32">
+        <f>IF($AD40=0,0,O40/(1-$AD40)-O40)</f>
+        <v/>
+      </c>
+      <c r="U40" s="33">
+        <f>O40+R40+S40+T40</f>
+        <v/>
+      </c>
+      <c r="V40" s="32">
+        <f>O40/(1-$C$8)-O40</f>
+        <v/>
+      </c>
+      <c r="W40" s="33">
+        <f>O40+V40</f>
+        <v/>
+      </c>
+      <c r="X40" s="32">
+        <f>O40/(1-$C$9)-O40</f>
+        <v/>
+      </c>
+      <c r="Y40" s="33">
+        <f>O40+X40</f>
+        <v/>
+      </c>
+      <c r="Z40" s="34">
+        <f>U40-Q40</f>
+        <v/>
+      </c>
+      <c r="AA40" s="34">
+        <f>W40-Q40</f>
+        <v/>
+      </c>
+      <c r="AB40" s="34">
+        <f>Y40-Q40</f>
+        <v/>
+      </c>
+      <c r="AD40" s="35" t="n">
         <v>0.06</v>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="43" t="n"/>
-      <c r="B40" s="44" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="43" t="n"/>
+      <c r="B41" s="44" t="inlineStr">
         <is>
           <t>Итого ИП МТ</t>
         </is>
       </c>
-      <c r="C40" s="43" t="n"/>
-      <c r="D40" s="43" t="n"/>
-      <c r="E40" s="43" t="n"/>
-      <c r="F40" s="43" t="n"/>
-      <c r="G40" s="43" t="n"/>
-      <c r="H40" s="43" t="n"/>
-      <c r="I40" s="45">
-        <f>SUM(I39:I39)</f>
-        <v/>
-      </c>
-      <c r="J40" s="45">
-        <f>SUM(J39:J39)</f>
-        <v/>
-      </c>
-      <c r="K40" s="45">
-        <f>SUM(K39:K39)</f>
-        <v/>
-      </c>
-      <c r="L40" s="45">
-        <f>SUM(L39:L39)</f>
-        <v/>
-      </c>
-      <c r="M40" s="45">
-        <f>SUM(M39:M39)</f>
-        <v/>
-      </c>
-      <c r="N40" s="45">
-        <f>SUM(N39:N39)</f>
-        <v/>
-      </c>
-      <c r="O40" s="45">
-        <f>SUM(O39:O39)</f>
-        <v/>
-      </c>
-      <c r="P40" s="45">
-        <f>SUM(P39:P39)</f>
-        <v/>
-      </c>
-      <c r="Q40" s="45">
-        <f>SUM(Q39:Q39)</f>
-        <v/>
-      </c>
-      <c r="R40" s="45">
-        <f>SUM(R39:R39)</f>
-        <v/>
-      </c>
-      <c r="S40" s="45">
-        <f>SUM(S39:S39)</f>
-        <v/>
-      </c>
-      <c r="T40" s="45">
-        <f>SUM(T39:T39)</f>
-        <v/>
-      </c>
-      <c r="U40" s="45">
-        <f>SUM(U39:U39)</f>
-        <v/>
-      </c>
-      <c r="V40" s="45">
-        <f>SUM(V39:V39)</f>
-        <v/>
-      </c>
-      <c r="W40" s="45">
-        <f>SUM(W39:W39)</f>
-        <v/>
-      </c>
-      <c r="X40" s="45">
-        <f>SUM(X39:X39)</f>
-        <v/>
-      </c>
-      <c r="Y40" s="45">
-        <f>SUM(Y39:Y39)</f>
-        <v/>
-      </c>
-      <c r="Z40" s="45">
-        <f>SUM(Z39:Z39)</f>
-        <v/>
-      </c>
-      <c r="AA40" s="45">
-        <f>SUM(AA39:AA39)</f>
-        <v/>
-      </c>
-      <c r="AB40" s="45">
-        <f>SUM(AB39:AB39)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="46" t="n"/>
-      <c r="B42" s="47" t="inlineStr">
-        <is>
-          <t>ВСЕГО (20 чел.)</t>
-        </is>
-      </c>
-      <c r="C42" s="46" t="n"/>
-      <c r="D42" s="46" t="n"/>
-      <c r="E42" s="46" t="n"/>
-      <c r="F42" s="46" t="n"/>
-      <c r="G42" s="46" t="n"/>
-      <c r="H42" s="46" t="n"/>
-      <c r="I42" s="48">
-        <f>I29+I36+I40</f>
-        <v/>
-      </c>
-      <c r="J42" s="48">
-        <f>J29+J36+J40</f>
-        <v/>
-      </c>
-      <c r="K42" s="48">
-        <f>K29+K36+K40</f>
-        <v/>
-      </c>
-      <c r="L42" s="48">
-        <f>L29+L36+L40</f>
-        <v/>
-      </c>
-      <c r="M42" s="48">
-        <f>M29+M36+M40</f>
-        <v/>
-      </c>
-      <c r="N42" s="48">
-        <f>N29+N36+N40</f>
-        <v/>
-      </c>
-      <c r="O42" s="48">
-        <f>O29+O36+O40</f>
-        <v/>
-      </c>
-      <c r="P42" s="48">
-        <f>P29+P36+P40</f>
-        <v/>
-      </c>
-      <c r="Q42" s="48">
-        <f>Q29+Q36+Q40</f>
-        <v/>
-      </c>
-      <c r="R42" s="48">
-        <f>R29+R36+R40</f>
-        <v/>
-      </c>
-      <c r="S42" s="48">
-        <f>S29+S36+S40</f>
-        <v/>
-      </c>
-      <c r="T42" s="48">
-        <f>T29+T36+T40</f>
-        <v/>
-      </c>
-      <c r="U42" s="48">
-        <f>U29+U36+U40</f>
-        <v/>
-      </c>
-      <c r="V42" s="48">
-        <f>V29+V36+V40</f>
-        <v/>
-      </c>
-      <c r="W42" s="48">
-        <f>W29+W36+W40</f>
-        <v/>
-      </c>
-      <c r="X42" s="48">
-        <f>X29+X36+X40</f>
-        <v/>
-      </c>
-      <c r="Y42" s="48">
-        <f>Y29+Y36+Y40</f>
-        <v/>
-      </c>
-      <c r="Z42" s="48">
-        <f>Z29+Z36+Z40</f>
-        <v/>
-      </c>
-      <c r="AA42" s="48">
-        <f>AA29+AA36+AA40</f>
-        <v/>
-      </c>
-      <c r="AB42" s="48">
-        <f>AB29+AB36+AB40</f>
-        <v/>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="49" t="inlineStr">
+      <c r="C41" s="43" t="n"/>
+      <c r="D41" s="43" t="n"/>
+      <c r="E41" s="43" t="n"/>
+      <c r="F41" s="43" t="n"/>
+      <c r="G41" s="43" t="n"/>
+      <c r="H41" s="43" t="n"/>
+      <c r="I41" s="45">
+        <f>SUM(I40:I40)</f>
+        <v/>
+      </c>
+      <c r="J41" s="45">
+        <f>SUM(J40:J40)</f>
+        <v/>
+      </c>
+      <c r="K41" s="45">
+        <f>SUM(K40:K40)</f>
+        <v/>
+      </c>
+      <c r="L41" s="45">
+        <f>SUM(L40:L40)</f>
+        <v/>
+      </c>
+      <c r="M41" s="45">
+        <f>SUM(M40:M40)</f>
+        <v/>
+      </c>
+      <c r="N41" s="45">
+        <f>SUM(N40:N40)</f>
+        <v/>
+      </c>
+      <c r="O41" s="45">
+        <f>SUM(O40:O40)</f>
+        <v/>
+      </c>
+      <c r="P41" s="45">
+        <f>SUM(P40:P40)</f>
+        <v/>
+      </c>
+      <c r="Q41" s="45">
+        <f>SUM(Q40:Q40)</f>
+        <v/>
+      </c>
+      <c r="R41" s="45">
+        <f>SUM(R40:R40)</f>
+        <v/>
+      </c>
+      <c r="S41" s="45">
+        <f>SUM(S40:S40)</f>
+        <v/>
+      </c>
+      <c r="T41" s="45">
+        <f>SUM(T40:T40)</f>
+        <v/>
+      </c>
+      <c r="U41" s="45">
+        <f>SUM(U40:U40)</f>
+        <v/>
+      </c>
+      <c r="V41" s="45">
+        <f>SUM(V40:V40)</f>
+        <v/>
+      </c>
+      <c r="W41" s="45">
+        <f>SUM(W40:W40)</f>
+        <v/>
+      </c>
+      <c r="X41" s="45">
+        <f>SUM(X40:X40)</f>
+        <v/>
+      </c>
+      <c r="Y41" s="45">
+        <f>SUM(Y40:Y40)</f>
+        <v/>
+      </c>
+      <c r="Z41" s="45">
+        <f>SUM(Z40:Z40)</f>
+        <v/>
+      </c>
+      <c r="AA41" s="45">
+        <f>SUM(AA40:AA40)</f>
+        <v/>
+      </c>
+      <c r="AB41" s="45">
+        <f>SUM(AB40:AB40)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="46" t="n"/>
+      <c r="B43" s="47" t="inlineStr">
+        <is>
+          <t>ВСЕГО (21 чел.)</t>
+        </is>
+      </c>
+      <c r="C43" s="46" t="n"/>
+      <c r="D43" s="46" t="n"/>
+      <c r="E43" s="46" t="n"/>
+      <c r="F43" s="46" t="n"/>
+      <c r="G43" s="46" t="n"/>
+      <c r="H43" s="46" t="n"/>
+      <c r="I43" s="48">
+        <f>I30+I37+I41</f>
+        <v/>
+      </c>
+      <c r="J43" s="48">
+        <f>J30+J37+J41</f>
+        <v/>
+      </c>
+      <c r="K43" s="48">
+        <f>K30+K37+K41</f>
+        <v/>
+      </c>
+      <c r="L43" s="48">
+        <f>L30+L37+L41</f>
+        <v/>
+      </c>
+      <c r="M43" s="48">
+        <f>M30+M37+M41</f>
+        <v/>
+      </c>
+      <c r="N43" s="48">
+        <f>N30+N37+N41</f>
+        <v/>
+      </c>
+      <c r="O43" s="48">
+        <f>O30+O37+O41</f>
+        <v/>
+      </c>
+      <c r="P43" s="48">
+        <f>P30+P37+P41</f>
+        <v/>
+      </c>
+      <c r="Q43" s="48">
+        <f>Q30+Q37+Q41</f>
+        <v/>
+      </c>
+      <c r="R43" s="48">
+        <f>R30+R37+R41</f>
+        <v/>
+      </c>
+      <c r="S43" s="48">
+        <f>S30+S37+S41</f>
+        <v/>
+      </c>
+      <c r="T43" s="48">
+        <f>T30+T37+T41</f>
+        <v/>
+      </c>
+      <c r="U43" s="48">
+        <f>U30+U37+U41</f>
+        <v/>
+      </c>
+      <c r="V43" s="48">
+        <f>V30+V37+V41</f>
+        <v/>
+      </c>
+      <c r="W43" s="48">
+        <f>W30+W37+W41</f>
+        <v/>
+      </c>
+      <c r="X43" s="48">
+        <f>X30+X37+X41</f>
+        <v/>
+      </c>
+      <c r="Y43" s="48">
+        <f>Y30+Y37+Y41</f>
+        <v/>
+      </c>
+      <c r="Z43" s="48">
+        <f>Z30+Z37+Z41</f>
+        <v/>
+      </c>
+      <c r="AA43" s="48">
+        <f>AA30+AA37+AA41</f>
+        <v/>
+      </c>
+      <c r="AB43" s="48">
+        <f>AB30+AB37+AB41</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="49" t="inlineStr">
         <is>
           <t>ПЛАНИРОВАНИЕ — сравнение схем</t>
         </is>
       </c>
     </row>
-    <row r="45" ht="32" customHeight="1">
-      <c r="A45" s="8" t="inlineStr">
+    <row r="46" ht="32" customHeight="1">
+      <c r="A46" s="7" t="inlineStr">
         <is>
           <t>Юр. лицо</t>
         </is>
       </c>
-      <c r="B45" s="8" t="inlineStr">
+      <c r="B46" s="7" t="inlineStr">
         <is>
           <t>Чел.</t>
         </is>
       </c>
-      <c r="C45" s="8" t="inlineStr">
+      <c r="C46" s="7" t="inlineStr">
         <is>
           <t>Напрямую: месяц</t>
         </is>
       </c>
-      <c r="D45" s="8" t="inlineStr">
+      <c r="D46" s="7" t="inlineStr">
         <is>
           <t>Напрямую: год</t>
         </is>
       </c>
-      <c r="E45" s="8" t="inlineStr">
+      <c r="E46" s="7" t="inlineStr">
         <is>
           <t>4dev: месяц</t>
         </is>
       </c>
-      <c r="F45" s="8" t="inlineStr">
+      <c r="F46" s="7" t="inlineStr">
         <is>
           <t>4dev: год</t>
         </is>
       </c>
-      <c r="G45" s="8" t="inlineStr">
+      <c r="G46" s="7" t="inlineStr">
         <is>
           <t>УСН 7%: месяц</t>
         </is>
       </c>
-      <c r="H45" s="8" t="inlineStr">
+      <c r="H46" s="7" t="inlineStr">
         <is>
           <t>УСН 7%: год</t>
         </is>
       </c>
-      <c r="I45" s="8" t="inlineStr">
+      <c r="I46" s="7" t="inlineStr">
         <is>
           <t>АУСН 8%: месяц</t>
         </is>
       </c>
-      <c r="J45" s="8" t="inlineStr">
+      <c r="J46" s="7" t="inlineStr">
         <is>
           <t>АУСН 8%: год</t>
         </is>
       </c>
-      <c r="K45" s="8" t="inlineStr">
+      <c r="K46" s="7" t="inlineStr">
         <is>
           <t>4dev − НПД за год</t>
         </is>
       </c>
-      <c r="L45" s="8" t="inlineStr">
+      <c r="L46" s="7" t="inlineStr">
         <is>
           <t>УСН − НПД за год</t>
         </is>
       </c>
-      <c r="M45" s="8" t="inlineStr">
+      <c r="M46" s="7" t="inlineStr">
         <is>
           <t>АУСН − НПД за год</t>
         </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="50" t="inlineStr">
-        <is>
-          <t>БВ</t>
-        </is>
-      </c>
-      <c r="B46" s="51" t="n">
-        <v>15</v>
-      </c>
-      <c r="C46" s="52">
-        <f>Q29</f>
-        <v/>
-      </c>
-      <c r="D46" s="53">
-        <f>Q29*12</f>
-        <v/>
-      </c>
-      <c r="E46" s="52">
-        <f>U29</f>
-        <v/>
-      </c>
-      <c r="F46" s="53">
-        <f>U29*12</f>
-        <v/>
-      </c>
-      <c r="G46" s="52">
-        <f>W29</f>
-        <v/>
-      </c>
-      <c r="H46" s="53">
-        <f>W29*12</f>
-        <v/>
-      </c>
-      <c r="I46" s="52">
-        <f>Y29</f>
-        <v/>
-      </c>
-      <c r="J46" s="53">
-        <f>Y29*12</f>
-        <v/>
-      </c>
-      <c r="K46" s="53">
-        <f>Z29*12</f>
-        <v/>
-      </c>
-      <c r="L46" s="53">
-        <f>AA29*12</f>
-        <v/>
-      </c>
-      <c r="M46" s="53">
-        <f>AB29*12</f>
-        <v/>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="50" t="inlineStr">
         <is>
-          <t>АС</t>
+          <t>БВ</t>
         </is>
       </c>
       <c r="B47" s="51" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="C47" s="52">
-        <f>Q36</f>
+        <f>Q30</f>
         <v/>
       </c>
       <c r="D47" s="53">
-        <f>Q36*12</f>
+        <f>Q30*12</f>
         <v/>
       </c>
       <c r="E47" s="52">
-        <f>U36</f>
+        <f>U30</f>
         <v/>
       </c>
       <c r="F47" s="53">
-        <f>U36*12</f>
+        <f>U30*12</f>
         <v/>
       </c>
       <c r="G47" s="52">
-        <f>W36</f>
+        <f>W30</f>
         <v/>
       </c>
       <c r="H47" s="53">
-        <f>W36*12</f>
+        <f>W30*12</f>
         <v/>
       </c>
       <c r="I47" s="52">
-        <f>Y36</f>
+        <f>Y30</f>
         <v/>
       </c>
       <c r="J47" s="53">
-        <f>Y36*12</f>
+        <f>Y30*12</f>
         <v/>
       </c>
       <c r="K47" s="53">
-        <f>Z36*12</f>
+        <f>Z30*12</f>
         <v/>
       </c>
       <c r="L47" s="53">
-        <f>AA36*12</f>
+        <f>AA30*12</f>
         <v/>
       </c>
       <c r="M47" s="53">
-        <f>AB36*12</f>
+        <f>AB30*12</f>
         <v/>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="50" t="inlineStr">
         <is>
+          <t>АС</t>
+        </is>
+      </c>
+      <c r="B48" s="51" t="n">
+        <v>4</v>
+      </c>
+      <c r="C48" s="52">
+        <f>Q37</f>
+        <v/>
+      </c>
+      <c r="D48" s="53">
+        <f>Q37*12</f>
+        <v/>
+      </c>
+      <c r="E48" s="52">
+        <f>U37</f>
+        <v/>
+      </c>
+      <c r="F48" s="53">
+        <f>U37*12</f>
+        <v/>
+      </c>
+      <c r="G48" s="52">
+        <f>W37</f>
+        <v/>
+      </c>
+      <c r="H48" s="53">
+        <f>W37*12</f>
+        <v/>
+      </c>
+      <c r="I48" s="52">
+        <f>Y37</f>
+        <v/>
+      </c>
+      <c r="J48" s="53">
+        <f>Y37*12</f>
+        <v/>
+      </c>
+      <c r="K48" s="53">
+        <f>Z37*12</f>
+        <v/>
+      </c>
+      <c r="L48" s="53">
+        <f>AA37*12</f>
+        <v/>
+      </c>
+      <c r="M48" s="53">
+        <f>AB37*12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="50" t="inlineStr">
+        <is>
           <t>ИП МТ</t>
         </is>
       </c>
-      <c r="B48" s="51" t="n">
+      <c r="B49" s="51" t="n">
         <v>1</v>
       </c>
-      <c r="C48" s="52">
-        <f>Q40</f>
-        <v/>
-      </c>
-      <c r="D48" s="53">
-        <f>Q40*12</f>
-        <v/>
-      </c>
-      <c r="E48" s="52">
-        <f>U40</f>
-        <v/>
-      </c>
-      <c r="F48" s="53">
-        <f>U40*12</f>
-        <v/>
-      </c>
-      <c r="G48" s="52">
-        <f>W40</f>
-        <v/>
-      </c>
-      <c r="H48" s="53">
-        <f>W40*12</f>
-        <v/>
-      </c>
-      <c r="I48" s="52">
-        <f>Y40</f>
-        <v/>
-      </c>
-      <c r="J48" s="53">
-        <f>Y40*12</f>
-        <v/>
-      </c>
-      <c r="K48" s="53">
-        <f>Z40*12</f>
-        <v/>
-      </c>
-      <c r="L48" s="53">
-        <f>AA40*12</f>
-        <v/>
-      </c>
-      <c r="M48" s="53">
-        <f>AB40*12</f>
-        <v/>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="54" t="inlineStr">
+      <c r="C49" s="52">
+        <f>Q41</f>
+        <v/>
+      </c>
+      <c r="D49" s="53">
+        <f>Q41*12</f>
+        <v/>
+      </c>
+      <c r="E49" s="52">
+        <f>U41</f>
+        <v/>
+      </c>
+      <c r="F49" s="53">
+        <f>U41*12</f>
+        <v/>
+      </c>
+      <c r="G49" s="52">
+        <f>W41</f>
+        <v/>
+      </c>
+      <c r="H49" s="53">
+        <f>W41*12</f>
+        <v/>
+      </c>
+      <c r="I49" s="52">
+        <f>Y41</f>
+        <v/>
+      </c>
+      <c r="J49" s="53">
+        <f>Y41*12</f>
+        <v/>
+      </c>
+      <c r="K49" s="53">
+        <f>Z41*12</f>
+        <v/>
+      </c>
+      <c r="L49" s="53">
+        <f>AA41*12</f>
+        <v/>
+      </c>
+      <c r="M49" s="53">
+        <f>AB41*12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="54" t="inlineStr">
         <is>
           <t>ИТОГО</t>
         </is>
       </c>
-      <c r="B49" s="55" t="n">
-        <v>20</v>
-      </c>
-      <c r="C49" s="56">
-        <f>Q42</f>
-        <v/>
-      </c>
-      <c r="D49" s="56">
-        <f>Q42*12</f>
-        <v/>
-      </c>
-      <c r="E49" s="56">
-        <f>U42</f>
-        <v/>
-      </c>
-      <c r="F49" s="56">
-        <f>U42*12</f>
-        <v/>
-      </c>
-      <c r="G49" s="56">
-        <f>W42</f>
-        <v/>
-      </c>
-      <c r="H49" s="56">
-        <f>W42*12</f>
-        <v/>
-      </c>
-      <c r="I49" s="56">
-        <f>Y42</f>
-        <v/>
-      </c>
-      <c r="J49" s="56">
-        <f>Y42*12</f>
-        <v/>
-      </c>
-      <c r="K49" s="56">
-        <f>Z42*12</f>
-        <v/>
-      </c>
-      <c r="L49" s="56">
-        <f>AA42*12</f>
-        <v/>
-      </c>
-      <c r="M49" s="56">
-        <f>AB42*12</f>
-        <v/>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="57" t="inlineStr">
+      <c r="B50" s="55" t="n">
+        <v>21</v>
+      </c>
+      <c r="C50" s="56">
+        <f>Q43</f>
+        <v/>
+      </c>
+      <c r="D50" s="56">
+        <f>Q43*12</f>
+        <v/>
+      </c>
+      <c r="E50" s="56">
+        <f>U43</f>
+        <v/>
+      </c>
+      <c r="F50" s="56">
+        <f>U43*12</f>
+        <v/>
+      </c>
+      <c r="G50" s="56">
+        <f>W43</f>
+        <v/>
+      </c>
+      <c r="H50" s="56">
+        <f>W43*12</f>
+        <v/>
+      </c>
+      <c r="I50" s="56">
+        <f>Y43</f>
+        <v/>
+      </c>
+      <c r="J50" s="56">
+        <f>Y43*12</f>
+        <v/>
+      </c>
+      <c r="K50" s="56">
+        <f>Z43*12</f>
+        <v/>
+      </c>
+      <c r="L50" s="56">
+        <f>AA43*12</f>
+        <v/>
+      </c>
+      <c r="M50" s="56">
+        <f>AB43*12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="57" t="inlineStr">
         <is>
           <t>Примечания</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="2" t="inlineStr">
-        <is>
-          <t>1. База «Среднемес. на руки 2026» = «Итого 2026» ÷ 7 × (1 − ставка НПД). Ставка НПД по каждому — столбец E (у Абдуллиной 0%).</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>2. «Напрямую самозанятому» — базовый вариант: на руки + НПД, без комиссии и сбора. Все разницы считаются от него.</t>
+          <t>1. База «Среднемес. на руки 2026» = «Итого 2026» ÷ 7 × (1 − ставка НПД). Ставка НПД по каждому — столбец E (у Абдуллиной 0%).</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>3. «Через площадку 4dev» — действующая схема: на руки + комиссия 3% + сбор ЮЛ Сингапура (÷0,975) + НПД.</t>
+          <t>2. «Напрямую самозанятому» — базовый вариант: на руки + НПД, без комиссии и сбора. Все разницы считаются от него.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>4. «ИП на УСН 7%» и «ИП на АУСН 8%» — гипотетические сценарии: те же суммы на руки, налог сверху (выплата = на руки ÷ (1 − ставка)).</t>
+          <t>3. «Через площадку 4dev» — действующая схема: на руки + комиссия 3% + сбор ЮЛ Сингапура (÷0,975) + НПД.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>5. Суммы по годам включают все типы начислений: ЗП, аутсорс и прочее. Устранено задвоение строк между листами-копиями.</t>
+          <t>4. «ИП на УСН 7%» и «ИП на АУСН 8%» — гипотетические сценарии: те же суммы на руки, налог сверху (выплата = на руки ÷ (1 − ставка)).</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>6. ОРАНЖЕВЫЕ ЯЧЕЙКИ в столбцах 2022–2026 собраны по отдельным строкам выплат — годовая сводная по этим людям в выгрузку Google Drive API не попала (она обрывается на фамилии «Косых»). Эти суммы могут быть занижены; сверьте их в исходной таблице.</t>
+          <t>5. Суммы по годам включают все типы начислений: ЗП, аутсорс и прочее. Устранено задвоение строк между листами-копиями.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Затронуты: Глубокая Яна Ярославовна — 2026; Жиркова Валентина Александровна — 2026; Оглезнева Полина Сергеевна — 2023; Оглезнева Полина Сергеевна — 2024; Оглезнева Полина Сергеевна — 2025; Нуруллина Анжелика Альбертовна — 2024; Нуруллина Анжелика Альбертовна — 2025; Кузнецова Светлана Дмитриевна — 2025; Кузьмина Елена Игоревна — 2023; Кузьмина Елена Игоревна — 2025; Левашева Анна Алексеевна — 2025; Лукьянова Вера Константиновна — 2024; Лукьянова Вера Константиновна — 2025; Тупико Олег Николаевич — 2024; Тупико Олег Николаевич — 2025; Репетенко Инна Эдуардовна — 2022; Репетенко Инна Эдуардовна — 2023; Репетенко Инна Эдуардовна — 2024; Репетенко Инна Эдуардовна — 2025</t>
+          <t>6. ЗЕЛЁНЫЕ ЯЧЕЙКИ (2025) — суммы, переданные заказчиком, они заменили собранные по строкам. Затронуто 14 человек.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>7. На расчёт схем это НЕ влияет: база берётся только из 2026 года, а годовая сводная за 2026 выгрузилась полностью (96 человек).</t>
+          <t xml:space="preserve">   У Нуруллиной заказчик передал две суммы (827 767,00 и 640 266,00) — в таблице они сложены: 1 468 033,00.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>8. Страховые взносы ИП в таблице НЕ учтены. На УСН ИП платит их за себя дополнительно, на АУСН взносы за себя не уплачиваются.</t>
+          <t>7. ОРАНЖЕВЫЕ ЯЧЕЙКИ собраны по отдельным строкам выплат — годовая сводная по этим людям в выгрузку Google Drive API не попала (она обрывается на фамилии «Косых»). Эти суммы могут быть занижены; сверьте их в исходной таблице.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>9. У АУСН есть ограничения: лимит дохода, численность до 5 человек, счёт в уполномоченном банке, доступен не во всех регионах.</t>
+          <t xml:space="preserve">   Затронуты: Глубокая Яна Ярославовна — 2026; Жиркова Валентина Александровна — 2026; Оглезнева Полина Сергеевна — 2023; Оглезнева Полина Сергеевна — 2024; Нуруллина Анжелика Альбертовна — 2024; Кузьмина Елена Игоревна — 2023; Лукьянова Вера Константиновна — 2024; Тупико Олег Николаевич — 2024; Репетенко Инна Эдуардовна — 2022; Репетенко Инна Эдуардовна — 2023; Репетенко Инна Эдуардовна — 2024; Шультяева Елизавета Александровна — 2025</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>10. Все ставки — в ячейках C5:C9. При изменении любой пересчитывается вся таблица и блок планирования.</t>
+          <t>8. На расчёт схем это НЕ влияет: база берётся только из 2026 года, а годовая сводная за 2026 выгрузилась полностью (96 человек).</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>11. Левашева и Капустина получают выплаты 2 года (2025–2026) — под критерий «более 2 лет» не подходят, включены по отдельной просьбе.</t>
+          <t>9. Страховые взносы ИП в таблице НЕ учтены. На УСН ИП платит их за себя дополнительно, на АУСН взносы за себя не уплачиваются.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>10. У АУСН есть ограничения: лимит дохода, численность до 5 человек, счёт в уполномоченном банке, доступен не во всех регионах.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>11. Все ставки — в ячейках C5:C9. При изменении любой пересчитывается вся таблица и блок планирования.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>12. Левашева, Капустина и Шультяева получают выплаты 2 года (2025–2026) — под критерий «более 2 лет» не подходят, включены по отдельной просьбе.</t>
         </is>
       </c>
     </row>

</xml_diff>